<commit_message>
Add SHA256 hashes and remaining Checks to workbook.
</commit_message>
<xml_diff>
--- a/reports/JY-Audit-Workbook.xlsx
+++ b/reports/JY-Audit-Workbook.xlsx
@@ -416,7 +416,7 @@
 </file>
 
 <file path=xl/tables/table11.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="11" name="EvidenceTable" displayName="EvidenceTable" ref="A1:I20" headerRowCount="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="11" name="EvidenceTable" displayName="EvidenceTable" ref="A1:I21" headerRowCount="1">
   <autoFilter ref="A1:I4"/>
   <tableColumns count="9">
     <tableColumn id="1" name="증적ID"/>
@@ -1334,7 +1334,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:I20"/>
+  <dimension ref="A1:I21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1344,7 +1344,7 @@
     <col width="10" customWidth="1" min="5" max="5"/>
     <col width="64" customWidth="1" min="6" max="6"/>
     <col width="10" customWidth="1" min="7" max="7"/>
-    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="72" customWidth="1" min="8" max="8"/>
     <col width="10" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
@@ -1569,7 +1569,11 @@
         </is>
       </c>
       <c r="G6" s="3" t="n"/>
-      <c r="H6" s="3" t="n"/>
+      <c r="H6" s="3" t="inlineStr">
+        <is>
+          <t>733293C02E65F593DDDAB16B6CE7505BB7E843CD20A67042C7CE1B031F527338</t>
+        </is>
+      </c>
       <c r="I6" s="3" t="inlineStr">
         <is>
           <t>토큰 미저장. .example.test만</t>
@@ -1606,7 +1610,11 @@
         </is>
       </c>
       <c r="G7" s="3" t="n"/>
-      <c r="H7" s="3" t="n"/>
+      <c r="H7" s="3" t="inlineStr">
+        <is>
+          <t>1EE5DD42AF94A4A38EB62827DF3B659AA84E88AEAFA85334F5D618F8FFAB0224</t>
+        </is>
+      </c>
       <c r="I7" s="3" t="inlineStr">
         <is>
           <t>S05 active=false</t>
@@ -1643,7 +1651,11 @@
         </is>
       </c>
       <c r="G8" s="3" t="n"/>
-      <c r="H8" s="3" t="n"/>
+      <c r="H8" s="3" t="inlineStr">
+        <is>
+          <t>11ECA98BE3060702DA44A8DB353F0F54A57DEFDA2C15DB308E3E1D54CB04957D</t>
+        </is>
+      </c>
       <c r="I8" s="3" t="inlineStr">
         <is>
           <t>합성 계정</t>
@@ -1680,7 +1692,11 @@
         </is>
       </c>
       <c r="G9" s="3" t="n"/>
-      <c r="H9" s="3" t="n"/>
+      <c r="H9" s="3" t="inlineStr">
+        <is>
+          <t>E0E8F4B36B38F969BA39BD63E96D07343D0886F253C5982F5560C648B3860A68</t>
+        </is>
+      </c>
       <c r="I9" s="3" t="inlineStr">
         <is>
           <t>합성 계정</t>
@@ -1717,7 +1733,11 @@
         </is>
       </c>
       <c r="G10" s="3" t="n"/>
-      <c r="H10" s="3" t="n"/>
+      <c r="H10" s="3" t="inlineStr">
+        <is>
+          <t>BB5D1CB3C45C6BF486506FA5D6E539C02502BD080D5AF54B8D7E3CD9509C932C</t>
+        </is>
+      </c>
       <c r="I10" s="3" t="inlineStr">
         <is>
           <t>T11 id=29 number=52028</t>
@@ -1754,7 +1774,11 @@
         </is>
       </c>
       <c r="G11" s="3" t="n"/>
-      <c r="H11" s="3" t="n"/>
+      <c r="H11" s="3" t="inlineStr">
+        <is>
+          <t>E59E461108AFCA1876D9391731187A1EFBA1F1073BF3789FB0D7168A6E801C54</t>
+        </is>
+      </c>
       <c r="I11" s="3" t="inlineStr">
         <is>
           <t>합성 계정</t>
@@ -1791,7 +1815,11 @@
         </is>
       </c>
       <c r="G12" s="3" t="n"/>
-      <c r="H12" s="3" t="n"/>
+      <c r="H12" s="3" t="inlineStr">
+        <is>
+          <t>24AA3EBEAE227353E9DE1E545987A30F133F1B814DE7AA09F34037563644AC50</t>
+        </is>
+      </c>
       <c r="I12" s="3" t="inlineStr">
         <is>
           <t>InPrivate</t>
@@ -1828,7 +1856,11 @@
         </is>
       </c>
       <c r="G13" s="3" t="n"/>
-      <c r="H13" s="3" t="n"/>
+      <c r="H13" s="3" t="inlineStr">
+        <is>
+          <t>820E8D35E734B01665B54B1F9F22E9809B25C1F1F24907C3A204BCE2A4F72B9C</t>
+        </is>
+      </c>
       <c r="I13" s="3" t="inlineStr">
         <is>
           <t>T11 id=29</t>
@@ -1838,7 +1870,7 @@
     <row r="14" ht="48" customHeight="1">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>E-F02-A02</t>
+          <t>E-F02-A01b</t>
         </is>
       </c>
       <c r="B14" s="10" t="n">
@@ -1851,7 +1883,7 @@
       </c>
       <c r="D14" s="3" t="inlineStr">
         <is>
-          <t>S04 T02 유지</t>
+          <t>S04 T11 권한 없음(T02 탭 포함)</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
@@ -1861,21 +1893,25 @@
       </c>
       <c r="F14" s="3" t="inlineStr">
         <is>
-          <t>C:\JY-Lab\private-evidence\after\E-F02-A02-S04-T02-ok.png</t>
+          <t>C:\JY-Lab\private-evidence\after\E-F02-A01-S04-T11-denied-T02tab.png</t>
         </is>
       </c>
       <c r="G14" s="3" t="n"/>
-      <c r="H14" s="3" t="n"/>
+      <c r="H14" s="3" t="inlineStr">
+        <is>
+          <t>47F8F8473CDF75BEA008F2A673430AC2601E154AADA4F4988196BA1E8C2BB2C6</t>
+        </is>
+      </c>
       <c r="I14" s="3" t="inlineStr">
         <is>
-          <t>T02 id=3 number=52003</t>
+          <t>A01 보조. 동일 세션 T02 탭</t>
         </is>
       </c>
     </row>
     <row r="15" ht="48" customHeight="1">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>E-F02-A03</t>
+          <t>E-F02-A02</t>
         </is>
       </c>
       <c r="B15" s="10" t="n">
@@ -1888,7 +1924,7 @@
       </c>
       <c r="D15" s="3" t="inlineStr">
         <is>
-          <t>C02 내 조직에서 T01 없음</t>
+          <t>S04 T02 유지</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
@@ -1898,21 +1934,25 @@
       </c>
       <c r="F15" s="3" t="inlineStr">
         <is>
-          <t>C:\JY-Lab\private-evidence\after\E-F02-A03-C02-no-T01.png</t>
+          <t>C:\JY-Lab\private-evidence\after\E-F02-A02-S04-T02-ok.png</t>
         </is>
       </c>
       <c r="G15" s="3" t="n"/>
-      <c r="H15" s="3" t="n"/>
+      <c r="H15" s="3" t="inlineStr">
+        <is>
+          <t>A1A72FAC7D94227E05261979A13A2E1DE81BF2B6800901B0492AD8EBADEF8A79</t>
+        </is>
+      </c>
       <c r="I15" s="3" t="inlineStr">
         <is>
-          <t>InPrivate</t>
+          <t>T02 id=3 number=52003</t>
         </is>
       </c>
     </row>
     <row r="16" ht="48" customHeight="1">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>E-F03-B01</t>
+          <t>E-F02-A03</t>
         </is>
       </c>
       <c r="B16" s="10" t="n">
@@ -1925,7 +1965,7 @@
       </c>
       <c r="D16" s="3" t="inlineStr">
         <is>
-          <t>C01 자료 보안 미리보기</t>
+          <t>C02 내 조직에서 T01 없음</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
@@ -1935,21 +1975,25 @@
       </c>
       <c r="F16" s="3" t="inlineStr">
         <is>
-          <t>C:\JY-Lab\private-evidence\before\E-F03-B01-C01-preview.png</t>
+          <t>C:\JY-Lab\private-evidence\after\E-F02-A03-C02-no-T01.png</t>
         </is>
       </c>
       <c r="G16" s="3" t="n"/>
-      <c r="H16" s="3" t="n"/>
+      <c r="H16" s="3" t="inlineStr">
+        <is>
+          <t>56F7E61008C2ED480A37A9499F4B2F20125BBE7DBD53E81ECBF5569B653FDD1C</t>
+        </is>
+      </c>
       <c r="I16" s="3" t="inlineStr">
         <is>
-          <t>T01·T11 4건. T12·T15 없음</t>
+          <t>InPrivate</t>
         </is>
       </c>
     </row>
     <row r="17" ht="48" customHeight="1">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>E-F03-B02</t>
+          <t>E-F03-B01</t>
         </is>
       </c>
       <c r="B17" s="10" t="n">
@@ -1962,7 +2006,7 @@
       </c>
       <c r="D17" s="3" t="inlineStr">
         <is>
-          <t>T12 삭제 전 마커</t>
+          <t>C01 자료 보안 미리보기</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
@@ -1972,21 +2016,25 @@
       </c>
       <c r="F17" s="3" t="inlineStr">
         <is>
-          <t>C:\JY-Lab\private-evidence\before\E-F03-B02-T12-marker.png</t>
+          <t>C:\JY-Lab\private-evidence\before\E-F03-B01-C01-preview.png</t>
         </is>
       </c>
       <c r="G17" s="3" t="n"/>
-      <c r="H17" s="3" t="n"/>
+      <c r="H17" s="3" t="inlineStr">
+        <is>
+          <t>DFBD99CD39F5B3F0B3068EEC58EEA47E1473413DDD72AB44F0FA6379AAD8DA2E</t>
+        </is>
+      </c>
       <c r="I17" s="3" t="inlineStr">
         <is>
-          <t>T12 id=14 number=52014</t>
+          <t>T01·T11 4건. T12·T15 없음</t>
         </is>
       </c>
     </row>
     <row r="18" ht="48" customHeight="1">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>E-F03-B03</t>
+          <t>E-F03-B02</t>
         </is>
       </c>
       <c r="B18" s="10" t="n">
@@ -1999,7 +2047,7 @@
       </c>
       <c r="D18" s="3" t="inlineStr">
         <is>
-          <t>T15 대조 삭제 전</t>
+          <t>T12 삭제 전 마커</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
@@ -2009,21 +2057,25 @@
       </c>
       <c r="F18" s="3" t="inlineStr">
         <is>
-          <t>C:\JY-Lab\private-evidence\before\E-F03-B03-T15-control.png</t>
+          <t>C:\JY-Lab\private-evidence\before\E-F03-B02-T12-marker.png</t>
         </is>
       </c>
       <c r="G18" s="3" t="n"/>
-      <c r="H18" s="3" t="n"/>
+      <c r="H18" s="3" t="inlineStr">
+        <is>
+          <t>E6B1424A80D6A20581D38278D80D12CBCA3225DB4B9AC67A61526582624B9B46</t>
+        </is>
+      </c>
       <c r="I18" s="3" t="inlineStr">
         <is>
-          <t>T15 id=17 number=52017</t>
+          <t>T12 id=14 number=52014</t>
         </is>
       </c>
     </row>
     <row r="19" ht="48" customHeight="1">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>E-F03-A01</t>
+          <t>E-F03-B03</t>
         </is>
       </c>
       <c r="B19" s="10" t="n">
@@ -2036,7 +2088,7 @@
       </c>
       <c r="D19" s="3" t="inlineStr">
         <is>
-          <t>T12 삭제 후 잔존</t>
+          <t>T15 대조 삭제 전</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
@@ -2046,21 +2098,25 @@
       </c>
       <c r="F19" s="3" t="inlineStr">
         <is>
-          <t>C:\JY-Lab\private-evidence\after\E-F03-A01-T12-residual.png</t>
+          <t>C:\JY-Lab\private-evidence\before\E-F03-B03-T15-control.png</t>
         </is>
       </c>
       <c r="G19" s="3" t="n"/>
-      <c r="H19" s="3" t="n"/>
+      <c r="H19" s="3" t="inlineStr">
+        <is>
+          <t>3BA3ED20A657A2AC4CB8336F3474531F7F997301E7DDFC9765A01FC75CA14C3C</t>
+        </is>
+      </c>
       <c r="I19" s="3" t="inlineStr">
         <is>
-          <t>C01 삭제 후 마커 잔존</t>
+          <t>T15 id=17 number=52017</t>
         </is>
       </c>
     </row>
     <row r="20" ht="48" customHeight="1">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>E-F03-A02</t>
+          <t>E-F03-A01</t>
         </is>
       </c>
       <c r="B20" s="10" t="n">
@@ -2073,22 +2129,67 @@
       </c>
       <c r="D20" s="3" t="inlineStr">
         <is>
+          <t>T12 삭제 후 잔존</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>화면</t>
+        </is>
+      </c>
+      <c r="F20" s="3" t="inlineStr">
+        <is>
+          <t>C:\JY-Lab\private-evidence\after\E-F03-A01-T12-residual.png</t>
+        </is>
+      </c>
+      <c r="G20" s="3" t="n"/>
+      <c r="H20" s="3" t="inlineStr">
+        <is>
+          <t>0C878A3FBCDEA9D5D7DD5EA3E1A3B3964E5040CFCE49F4460F976EAB10ECDD23</t>
+        </is>
+      </c>
+      <c r="I20" s="3" t="inlineStr">
+        <is>
+          <t>C01 삭제 후 마커 잔존</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="48" customHeight="1">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>E-F03-A02</t>
+        </is>
+      </c>
+      <c r="B21" s="10" t="n">
+        <v>46301</v>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>수행자</t>
+        </is>
+      </c>
+      <c r="D21" s="3" t="inlineStr">
+        <is>
           <t>T15 삭제 후 보존</t>
         </is>
       </c>
-      <c r="E20" s="2" t="inlineStr">
+      <c r="E21" s="2" t="inlineStr">
         <is>
           <t>화면</t>
         </is>
       </c>
-      <c r="F20" s="3" t="inlineStr">
+      <c r="F21" s="3" t="inlineStr">
         <is>
           <t>C:\JY-Lab\private-evidence\after\E-F03-A02-T15-preserved.png</t>
         </is>
       </c>
-      <c r="G20" s="3" t="n"/>
-      <c r="H20" s="3" t="n"/>
-      <c r="I20" s="3" t="inlineStr">
+      <c r="G21" s="3" t="n"/>
+      <c r="H21" s="3" t="inlineStr">
+        <is>
+          <t>5B576280C64B3E30B77034CBE4A37E40DDBB166FBFF2BEAF33FDE7DC3708A553</t>
+        </is>
+      </c>
+      <c r="I21" s="3" t="inlineStr">
         <is>
           <t>대조 티켓 보존</t>
         </is>
@@ -3306,7 +3407,7 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="36" customHeight="1">
+    <row r="2" ht="48" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>A01</t>
@@ -3329,26 +3430,26 @@
       </c>
       <c r="E2" s="3" t="inlineStr">
         <is>
-          <t>scope.md 작성</t>
+          <t>docs/scope.md.txt와 localhost:8080 대조. 3조직 1시스템, 결제·배송·마케팅·백업 실측 제외.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>미실시</t>
+          <t>적합</t>
         </is>
       </c>
       <c r="G2" s="3" t="inlineStr">
         <is>
-          <t>scope.md</t>
+          <t>docs/scope.md.txt</t>
         </is>
       </c>
       <c r="H2" s="3" t="inlineStr">
         <is>
-          <t>모의와 실제 구별</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="36" customHeight="1">
+          <t>모의와 실제 구별. 범위 문서 기준.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="48" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
           <t>A02</t>
@@ -3371,26 +3472,26 @@
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>sources.csv 완료</t>
+          <t>docs/sources.csv에 법령·시행령·고시·처리방침 지침 시행일·확인일(2026-09-21) 기록.</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>미실시</t>
+          <t>적합</t>
         </is>
       </c>
       <c r="G3" s="3" t="inlineStr">
         <is>
-          <t>S-L01</t>
+          <t>S-L01~S-L04</t>
         </is>
       </c>
       <c r="H3" s="3" t="inlineStr">
         <is>
-          <t>AI조문 금지</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="36" customHeight="1">
+          <t>AI 생성 조문 미사용. 항·호는 원문 추가분만 Controls.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="48" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
           <t>A03</t>
@@ -3413,26 +3514,26 @@
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>data-flow.pdf</t>
+          <t>docs/data-flow.pdf에 티켓·첨부·백업(점선) 경로 표시.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>미실시</t>
+          <t>적합</t>
         </is>
       </c>
       <c r="G4" s="3" t="inlineStr">
         <is>
-          <t>data-flow.pdf</t>
+          <t>DF-01</t>
         </is>
       </c>
       <c r="H4" s="3" t="inlineStr">
         <is>
-          <t>백업 점선</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="36" customHeight="1">
+          <t>논리흐름. 백업 실측 아님.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="48" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
         <is>
           <t>A04</t>
@@ -3455,26 +3556,26 @@
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>interview.md</t>
+          <t>docs/interview.md.txt에 발급·종료·파기 역할 질문. 시스템 Admin은 S01, 문서상 책임은 S02.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>미실시</t>
+          <t>적합</t>
         </is>
       </c>
       <c r="G5" s="3" t="inlineStr">
         <is>
-          <t>interview.md</t>
+          <t>docs/interview.md.txt</t>
         </is>
       </c>
       <c r="H5" s="3" t="inlineStr">
         <is>
-          <t>실제 조직운영 미확인</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="36" customHeight="1">
+          <t>실제 조직 운영·서명은 미확인.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="48" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
           <t>B01</t>
@@ -3497,22 +3598,26 @@
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>이름이메일문의첨부</t>
+          <t>상담 항목은 이름·이메일·문의·첨부. 합성자료에 주민번호·민감정보 없음.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>미실시</t>
-        </is>
-      </c>
-      <c r="G6" s="3" t="n"/>
+          <t>적합</t>
+        </is>
+      </c>
+      <c r="G6" s="3" t="inlineStr">
+        <is>
+          <t>tickets.csv, control-notes.md</t>
+        </is>
+      </c>
       <c r="H6" s="3" t="inlineStr">
         <is>
-          <t>주민번호 없음</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="36" customHeight="1">
+          <t>목적별 세분 고지는 티켓 양식에 없음.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="48" customHeight="1">
       <c r="A7" s="2" t="inlineStr">
         <is>
           <t>B02</t>
@@ -3535,22 +3640,26 @@
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>처리방침 미흡 설정</t>
+          <t>docs/client-before/02-privacy-policy.md.txt는 보유·위탁·권리가 초기 미흡 설정.</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>미실시</t>
+          <t>미흡</t>
         </is>
       </c>
       <c r="G7" s="3" t="inlineStr">
         <is>
-          <t>02-privacy-policy.md</t>
-        </is>
-      </c>
-      <c r="H7" s="3" t="n"/>
-    </row>
-    <row r="8" ht="36" customHeight="1">
+          <t>02-privacy-policy.md.txt</t>
+        </is>
+      </c>
+      <c r="H7" s="3" t="inlineStr">
+        <is>
+          <t>운영(Zammad)과 방침 문구 불일치 가능.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="48" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
           <t>B03</t>
@@ -3573,22 +3682,26 @@
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>01·03문서</t>
+          <t>01·03 문서에 Retail 목적, Service 상담, Vendor 유지보수는 있으나 제공·위탁 구분이 빈약.</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>미실시</t>
+          <t>미흡</t>
         </is>
       </c>
       <c r="G8" s="3" t="inlineStr">
         <is>
-          <t>03-outsourcing.md</t>
-        </is>
-      </c>
-      <c r="H8" s="3" t="n"/>
-    </row>
-    <row r="9" ht="36" customHeight="1">
+          <t>03-outsourcing.md.txt</t>
+        </is>
+      </c>
+      <c r="H8" s="3" t="inlineStr">
+        <is>
+          <t>연간 수탁 점검은 D01.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="48" customHeight="1">
       <c r="A9" s="2" t="inlineStr">
         <is>
           <t>B04</t>
@@ -3611,22 +3724,26 @@
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>13장 전</t>
+          <t>C01 삭제는 자료 보안으로 실행. 접수·본인확인·회신 메일 흐름은 없음.</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>미실시</t>
-        </is>
-      </c>
-      <c r="G9" s="3" t="n"/>
+          <t>미확인</t>
+        </is>
+      </c>
+      <c r="G9" s="3" t="inlineStr">
+        <is>
+          <t>E-F03-B01</t>
+        </is>
+      </c>
       <c r="H9" s="3" t="inlineStr">
         <is>
-          <t>실제 발송 없음</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="36" customHeight="1">
+          <t>실제 발송 없음. 권리 절차 문서는 초기자료에 없음.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="48" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
         <is>
           <t>C01</t>
@@ -3649,20 +3766,24 @@
       </c>
       <c r="E10" s="3" t="inlineStr">
         <is>
-          <t>S01만 Admin</t>
+          <t>직원 6명 명부·Accounts 대조. Admin은 S01만. 이메일은 .example.test.</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>미실시</t>
+          <t>적합</t>
         </is>
       </c>
       <c r="G10" s="3" t="inlineStr">
         <is>
-          <t>Accounts</t>
-        </is>
-      </c>
-      <c r="H10" s="3" t="n"/>
+          <t>Accounts, staff.csv</t>
+        </is>
+      </c>
+      <c r="H10" s="3" t="inlineStr">
+        <is>
+          <t>가상 명부. 실명 인사시스템 없음.</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="48" customHeight="1">
       <c r="A11" s="2" t="inlineStr">
@@ -3790,7 +3911,7 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="36" customHeight="1">
+    <row r="14" ht="48" customHeight="1">
       <c r="A14" s="2" t="inlineStr">
         <is>
           <t>D01</t>
@@ -3813,22 +3934,22 @@
       </c>
       <c r="E14" s="3" t="inlineStr">
         <is>
-          <t>03문서 빈약</t>
+          <t>03-outsourcing.md.txt에 계약·점검표·연간실적 없음.</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>미실시</t>
+          <t>미흡</t>
         </is>
       </c>
       <c r="G14" s="3" t="inlineStr">
         <is>
-          <t>03-outsourcing.md</t>
+          <t>03-outsourcing.md.txt</t>
         </is>
       </c>
       <c r="H14" s="3" t="inlineStr">
         <is>
-          <t>연간실적 없음</t>
+          <t>수탁 감독 실적은 문서상 확인 불가.</t>
         </is>
       </c>
     </row>
@@ -3874,7 +3995,7 @@
         </is>
       </c>
     </row>
-    <row r="16" ht="36" customHeight="1">
+    <row r="16" ht="48" customHeight="1">
       <c r="A16" s="2" t="inlineStr">
         <is>
           <t>D03</t>
@@ -3897,22 +4018,22 @@
       </c>
       <c r="E16" s="3" t="inlineStr">
         <is>
-          <t>13장 전</t>
+          <t>jy-doc02 등 다운로드 사본의 PC 위치·파기는 화면 미실측.</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>미실시</t>
+          <t>미확인</t>
         </is>
       </c>
       <c r="G16" s="3" t="n"/>
       <c r="H16" s="3" t="inlineStr">
         <is>
-          <t>권한회수로 사본은 안 지워짐</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="36" customHeight="1">
+          <t>권한 회수·사용자 삭제로 로컬 사본은 지워지지 않음.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="48" customHeight="1">
       <c r="A17" s="2" t="inlineStr">
         <is>
           <t>D04</t>
@@ -3935,22 +4056,22 @@
       </c>
       <c r="E17" s="3" t="inlineStr">
         <is>
-          <t>미작성</t>
+          <t>교육 1장·검토 양식 미작성. client-before에 교육 기록이 없음.</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>미실시</t>
+          <t>미흡</t>
         </is>
       </c>
       <c r="G17" s="3" t="n"/>
       <c r="H17" s="3" t="inlineStr">
         <is>
-          <t>장기 서명 없음</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="36" customHeight="1">
+          <t>장기 서명·이수 증빙 없음.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="48" customHeight="1">
       <c r="A18" s="2" t="inlineStr">
         <is>
           <t>E01</t>
@@ -3973,22 +4094,22 @@
       </c>
       <c r="E18" s="3" t="inlineStr">
         <is>
-          <t>필요할 때까지 모호</t>
+          <t>05-retention.md.txt·Processing 보유가 '필요할 때까지'로 모호. 기간·방법 불명확.</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>미실시</t>
+          <t>미흡</t>
         </is>
       </c>
       <c r="G18" s="3" t="inlineStr">
         <is>
-          <t>05-retention.md</t>
+          <t>05-retention.md.txt</t>
         </is>
       </c>
       <c r="H18" s="3" t="inlineStr">
         <is>
-          <t>임의 연수 금지</t>
+          <t>임의 연수 기재 금지. 원문 대조만.</t>
         </is>
       </c>
     </row>
@@ -4114,7 +4235,7 @@
         </is>
       </c>
     </row>
-    <row r="22" ht="36" customHeight="1">
+    <row r="22" ht="48" customHeight="1">
       <c r="A22" s="2" t="inlineStr">
         <is>
           <t>F01</t>
@@ -4137,12 +4258,12 @@
       </c>
       <c r="E22" s="3" t="inlineStr">
         <is>
-          <t>ENV 파일</t>
+          <t>F-01~F-03 화면·JSON SHA256 수집. 명부 이메일 .example.test. 토큰 미저장.</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>미실시</t>
+          <t>적합</t>
         </is>
       </c>
       <c r="G22" s="3" t="inlineStr">
@@ -4150,9 +4271,13 @@
           <t>Evidence</t>
         </is>
       </c>
-      <c r="H22" s="3" t="n"/>
-    </row>
-    <row r="23" ht="36" customHeight="1">
+      <c r="H22" s="3" t="inlineStr">
+        <is>
+          <t>ENV-01 등 환경 증적 해시는 미기입. 원본은 Git 밖.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="48" customHeight="1">
       <c r="A23" s="2" t="inlineStr">
         <is>
           <t>F02</t>
@@ -4175,22 +4300,26 @@
       </c>
       <c r="E23" s="3" t="inlineStr">
         <is>
-          <t>06문서 양식없음</t>
+          <t>06-incident.md.txt에 사고 양식·담당·통지 근거 없음. 도상훈련 미실시.</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>미실시</t>
-        </is>
-      </c>
-      <c r="G23" s="3" t="n"/>
+          <t>미흡</t>
+        </is>
+      </c>
+      <c r="G23" s="3" t="inlineStr">
+        <is>
+          <t>06-incident.md.txt</t>
+        </is>
+      </c>
       <c r="H23" s="3" t="inlineStr">
         <is>
-          <t>16장·실제 신고 안 함</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="36" customHeight="1">
+          <t>실제 신고·72시간 단순화 금지.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="48" customHeight="1">
       <c r="A24" s="2" t="inlineStr">
         <is>
           <t>F03</t>
@@ -4213,18 +4342,18 @@
       </c>
       <c r="E24" s="3" t="inlineStr">
         <is>
-          <t>외부 AI 미연결</t>
+          <t>외부 AI 요약도구 미연결. 제공자 조건 공란.</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>미실시</t>
+          <t>적용 제외</t>
         </is>
       </c>
       <c r="G24" s="3" t="n"/>
       <c r="H24" s="3" t="inlineStr">
         <is>
-          <t>16.3·공격시험 안 함</t>
+          <t>공격시험 안 함. 16.3 해당 시 별도.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Refresh audit workbook with D03 copy, users-diff, and session limits.
</commit_message>
<xml_diff>
--- a/reports/JY-Audit-Workbook.xlsx
+++ b/reports/JY-Audit-Workbook.xlsx
@@ -416,7 +416,7 @@
 </file>
 
 <file path=xl/tables/table11.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="11" name="EvidenceTable" displayName="EvidenceTable" ref="A1:I21" headerRowCount="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="11" name="EvidenceTable" displayName="EvidenceTable" ref="A1:I23" headerRowCount="1">
   <autoFilter ref="A1:I4"/>
   <tableColumns count="9">
     <tableColumn id="1" name="증적ID"/>
@@ -1300,7 +1300,7 @@
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>T12 마커·다운로드 사본·백업은 미파기</t>
+          <t>T12 마커·다운로드 사본(jy-doc02-copy.txt)·백업은 미파기</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
@@ -1334,7 +1334,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:I21"/>
+  <dimension ref="A1:I23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1624,7 +1624,7 @@
     <row r="8" ht="48" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>E-F01-B01</t>
+          <t>JSON-F01-DIFF</t>
         </is>
       </c>
       <c r="B8" s="10" t="n">
@@ -1637,35 +1637,31 @@
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>S05 T02 열람</t>
+          <t>Users 전후 비교</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>화면</t>
+          <t>파일</t>
         </is>
       </c>
       <c r="F8" s="3" t="inlineStr">
         <is>
-          <t>C:\JY-Lab\private-evidence\before\E-F01-B01-S05-active-T02.png</t>
+          <t>C:\JY-Lab\private-evidence\after\users-diff.json</t>
         </is>
       </c>
       <c r="G8" s="3" t="n"/>
-      <c r="H8" s="3" t="inlineStr">
-        <is>
-          <t>11ECA98BE3060702DA44A8DB353F0F54A57DEFDA2C15DB308E3E1D54CB04957D</t>
-        </is>
-      </c>
+      <c r="H8" s="3" t="n"/>
       <c r="I8" s="3" t="inlineStr">
         <is>
-          <t>합성 계정</t>
+          <t>S05 active True→False만 변경. Git 제외. SHA256은 로컬 Get-FileHash</t>
         </is>
       </c>
     </row>
     <row r="9" ht="48" customHeight="1">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>E-F01-A01</t>
+          <t>E-F01-B01</t>
         </is>
       </c>
       <c r="B9" s="10" t="n">
@@ -1678,7 +1674,7 @@
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>S05 로그인 차단</t>
+          <t>S05 T02 열람</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
@@ -1688,13 +1684,13 @@
       </c>
       <c r="F9" s="3" t="inlineStr">
         <is>
-          <t>C:\JY-Lab\private-evidence\after\E-F01-A01-S05-login-blocked.png</t>
+          <t>C:\JY-Lab\private-evidence\before\E-F01-B01-S05-active-T02.png</t>
         </is>
       </c>
       <c r="G9" s="3" t="n"/>
       <c r="H9" s="3" t="inlineStr">
         <is>
-          <t>E0E8F4B36B38F969BA39BD63E96D07343D0886F253C5982F5560C648B3860A68</t>
+          <t>11ECA98BE3060702DA44A8DB353F0F54A57DEFDA2C15DB308E3E1D54CB04957D</t>
         </is>
       </c>
       <c r="I9" s="3" t="inlineStr">
@@ -1706,7 +1702,7 @@
     <row r="10" ht="48" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>E-F02-B01</t>
+          <t>E-F01-A01</t>
         </is>
       </c>
       <c r="B10" s="10" t="n">
@@ -1719,7 +1715,7 @@
       </c>
       <c r="D10" s="3" t="inlineStr">
         <is>
-          <t>S04 T11 열람</t>
+          <t>S05 로그인 차단</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
@@ -1729,25 +1725,25 @@
       </c>
       <c r="F10" s="3" t="inlineStr">
         <is>
-          <t>C:\JY-Lab\private-evidence\before\E-F02-B01-S04-T11.png</t>
+          <t>C:\JY-Lab\private-evidence\after\E-F01-A01-S05-login-blocked.png</t>
         </is>
       </c>
       <c r="G10" s="3" t="n"/>
       <c r="H10" s="3" t="inlineStr">
         <is>
-          <t>BB5D1CB3C45C6BF486506FA5D6E539C02502BD080D5AF54B8D7E3CD9509C932C</t>
+          <t>E0E8F4B36B38F969BA39BD63E96D07343D0886F253C5982F5560C648B3860A68</t>
         </is>
       </c>
       <c r="I10" s="3" t="inlineStr">
         <is>
-          <t>T11 id=29 number=52028</t>
+          <t>합성 계정</t>
         </is>
       </c>
     </row>
     <row r="11" ht="48" customHeight="1">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>E-F02-B02</t>
+          <t>E-F02-B01</t>
         </is>
       </c>
       <c r="B11" s="10" t="n">
@@ -1760,7 +1756,7 @@
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
-          <t>S06 T11 열람</t>
+          <t>S04 T11 열람</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
@@ -1770,25 +1766,25 @@
       </c>
       <c r="F11" s="3" t="inlineStr">
         <is>
-          <t>C:\JY-Lab\private-evidence\before\E-F02-B02-S06-T11.png</t>
+          <t>C:\JY-Lab\private-evidence\before\E-F02-B01-S04-T11.png</t>
         </is>
       </c>
       <c r="G11" s="3" t="n"/>
       <c r="H11" s="3" t="inlineStr">
         <is>
-          <t>E59E461108AFCA1876D9391731187A1EFBA1F1073BF3789FB0D7168A6E801C54</t>
+          <t>BB5D1CB3C45C6BF486506FA5D6E539C02502BD080D5AF54B8D7E3CD9509C932C</t>
         </is>
       </c>
       <c r="I11" s="3" t="inlineStr">
         <is>
-          <t>합성 계정</t>
+          <t>T11 id=29 number=52028</t>
         </is>
       </c>
     </row>
     <row r="12" ht="48" customHeight="1">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>E-F02-B03</t>
+          <t>E-F02-B02</t>
         </is>
       </c>
       <c r="B12" s="10" t="n">
@@ -1801,7 +1797,7 @@
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>C02가 T01 열람</t>
+          <t>S06 T11 열람</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
@@ -1811,25 +1807,25 @@
       </c>
       <c r="F12" s="3" t="inlineStr">
         <is>
-          <t>C:\JY-Lab\private-evidence\before\E-F02-B03-C02-sees-T01.png</t>
+          <t>C:\JY-Lab\private-evidence\before\E-F02-B02-S06-T11.png</t>
         </is>
       </c>
       <c r="G12" s="3" t="n"/>
       <c r="H12" s="3" t="inlineStr">
         <is>
-          <t>24AA3EBEAE227353E9DE1E545987A30F133F1B814DE7AA09F34037563644AC50</t>
+          <t>E59E461108AFCA1876D9391731187A1EFBA1F1073BF3789FB0D7168A6E801C54</t>
         </is>
       </c>
       <c r="I12" s="3" t="inlineStr">
         <is>
-          <t>InPrivate</t>
+          <t>합성 계정</t>
         </is>
       </c>
     </row>
     <row r="13" ht="48" customHeight="1">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>E-F02-A01</t>
+          <t>E-F02-B03</t>
         </is>
       </c>
       <c r="B13" s="10" t="n">
@@ -1842,7 +1838,7 @@
       </c>
       <c r="D13" s="3" t="inlineStr">
         <is>
-          <t>S04 T11 권한 없음</t>
+          <t>C02가 T01 열람</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
@@ -1852,25 +1848,25 @@
       </c>
       <c r="F13" s="3" t="inlineStr">
         <is>
-          <t>C:\JY-Lab\private-evidence\after\E-F02-A01-S04-T11-denied.png</t>
+          <t>C:\JY-Lab\private-evidence\before\E-F02-B03-C02-sees-T01.png</t>
         </is>
       </c>
       <c r="G13" s="3" t="n"/>
       <c r="H13" s="3" t="inlineStr">
         <is>
-          <t>820E8D35E734B01665B54B1F9F22E9809B25C1F1F24907C3A204BCE2A4F72B9C</t>
+          <t>24AA3EBEAE227353E9DE1E545987A30F133F1B814DE7AA09F34037563644AC50</t>
         </is>
       </c>
       <c r="I13" s="3" t="inlineStr">
         <is>
-          <t>T11 id=29</t>
+          <t>InPrivate</t>
         </is>
       </c>
     </row>
     <row r="14" ht="48" customHeight="1">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>E-F02-A01b</t>
+          <t>E-F02-A01</t>
         </is>
       </c>
       <c r="B14" s="10" t="n">
@@ -1883,7 +1879,7 @@
       </c>
       <c r="D14" s="3" t="inlineStr">
         <is>
-          <t>S04 T11 권한 없음(T02 탭 포함)</t>
+          <t>S04 T11 권한 없음</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
@@ -1893,25 +1889,25 @@
       </c>
       <c r="F14" s="3" t="inlineStr">
         <is>
-          <t>C:\JY-Lab\private-evidence\after\E-F02-A01-S04-T11-denied-T02tab.png</t>
+          <t>C:\JY-Lab\private-evidence\after\E-F02-A01-S04-T11-denied.png</t>
         </is>
       </c>
       <c r="G14" s="3" t="n"/>
       <c r="H14" s="3" t="inlineStr">
         <is>
-          <t>47F8F8473CDF75BEA008F2A673430AC2601E154AADA4F4988196BA1E8C2BB2C6</t>
+          <t>820E8D35E734B01665B54B1F9F22E9809B25C1F1F24907C3A204BCE2A4F72B9C</t>
         </is>
       </c>
       <c r="I14" s="3" t="inlineStr">
         <is>
-          <t>A01 보조. 동일 세션 T02 탭</t>
+          <t>T11 id=29</t>
         </is>
       </c>
     </row>
     <row r="15" ht="48" customHeight="1">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>E-F02-A02</t>
+          <t>E-F02-A01b</t>
         </is>
       </c>
       <c r="B15" s="10" t="n">
@@ -1924,7 +1920,7 @@
       </c>
       <c r="D15" s="3" t="inlineStr">
         <is>
-          <t>S04 T02 유지</t>
+          <t>S04 T11 권한 없음(T02 탭 포함)</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
@@ -1934,25 +1930,25 @@
       </c>
       <c r="F15" s="3" t="inlineStr">
         <is>
-          <t>C:\JY-Lab\private-evidence\after\E-F02-A02-S04-T02-ok.png</t>
+          <t>C:\JY-Lab\private-evidence\after\E-F02-A01-S04-T11-denied-T02tab.png</t>
         </is>
       </c>
       <c r="G15" s="3" t="n"/>
       <c r="H15" s="3" t="inlineStr">
         <is>
-          <t>A1A72FAC7D94227E05261979A13A2E1DE81BF2B6800901B0492AD8EBADEF8A79</t>
+          <t>47F8F8473CDF75BEA008F2A673430AC2601E154AADA4F4988196BA1E8C2BB2C6</t>
         </is>
       </c>
       <c r="I15" s="3" t="inlineStr">
         <is>
-          <t>T02 id=3 number=52003</t>
+          <t>A01 보조. 동일 세션 T02 탭</t>
         </is>
       </c>
     </row>
     <row r="16" ht="48" customHeight="1">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>E-F02-A03</t>
+          <t>E-F02-A02</t>
         </is>
       </c>
       <c r="B16" s="10" t="n">
@@ -1965,7 +1961,7 @@
       </c>
       <c r="D16" s="3" t="inlineStr">
         <is>
-          <t>C02 내 조직에서 T01 없음</t>
+          <t>S04 T02 유지</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
@@ -1975,25 +1971,25 @@
       </c>
       <c r="F16" s="3" t="inlineStr">
         <is>
-          <t>C:\JY-Lab\private-evidence\after\E-F02-A03-C02-no-T01.png</t>
+          <t>C:\JY-Lab\private-evidence\after\E-F02-A02-S04-T02-ok.png</t>
         </is>
       </c>
       <c r="G16" s="3" t="n"/>
       <c r="H16" s="3" t="inlineStr">
         <is>
-          <t>56F7E61008C2ED480A37A9499F4B2F20125BBE7DBD53E81ECBF5569B653FDD1C</t>
+          <t>A1A72FAC7D94227E05261979A13A2E1DE81BF2B6800901B0492AD8EBADEF8A79</t>
         </is>
       </c>
       <c r="I16" s="3" t="inlineStr">
         <is>
-          <t>InPrivate</t>
+          <t>T02 id=3 number=52003</t>
         </is>
       </c>
     </row>
     <row r="17" ht="48" customHeight="1">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>E-F03-B01</t>
+          <t>E-F02-A03</t>
         </is>
       </c>
       <c r="B17" s="10" t="n">
@@ -2006,7 +2002,7 @@
       </c>
       <c r="D17" s="3" t="inlineStr">
         <is>
-          <t>C01 자료 보안 미리보기</t>
+          <t>C02 내 조직에서 T01 없음</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
@@ -2016,25 +2012,25 @@
       </c>
       <c r="F17" s="3" t="inlineStr">
         <is>
-          <t>C:\JY-Lab\private-evidence\before\E-F03-B01-C01-preview.png</t>
+          <t>C:\JY-Lab\private-evidence\after\E-F02-A03-C02-no-T01.png</t>
         </is>
       </c>
       <c r="G17" s="3" t="n"/>
       <c r="H17" s="3" t="inlineStr">
         <is>
-          <t>DFBD99CD39F5B3F0B3068EEC58EEA47E1473413DDD72AB44F0FA6379AAD8DA2E</t>
+          <t>56F7E61008C2ED480A37A9499F4B2F20125BBE7DBD53E81ECBF5569B653FDD1C</t>
         </is>
       </c>
       <c r="I17" s="3" t="inlineStr">
         <is>
-          <t>T01·T11 4건. T12·T15 없음</t>
+          <t>InPrivate</t>
         </is>
       </c>
     </row>
     <row r="18" ht="48" customHeight="1">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>E-F03-B02</t>
+          <t>E-F03-B01</t>
         </is>
       </c>
       <c r="B18" s="10" t="n">
@@ -2047,7 +2043,7 @@
       </c>
       <c r="D18" s="3" t="inlineStr">
         <is>
-          <t>T12 삭제 전 마커</t>
+          <t>C01 자료 보안 미리보기</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
@@ -2057,25 +2053,25 @@
       </c>
       <c r="F18" s="3" t="inlineStr">
         <is>
-          <t>C:\JY-Lab\private-evidence\before\E-F03-B02-T12-marker.png</t>
+          <t>C:\JY-Lab\private-evidence\before\E-F03-B01-C01-preview.png</t>
         </is>
       </c>
       <c r="G18" s="3" t="n"/>
       <c r="H18" s="3" t="inlineStr">
         <is>
-          <t>E6B1424A80D6A20581D38278D80D12CBCA3225DB4B9AC67A61526582624B9B46</t>
+          <t>DFBD99CD39F5B3F0B3068EEC58EEA47E1473413DDD72AB44F0FA6379AAD8DA2E</t>
         </is>
       </c>
       <c r="I18" s="3" t="inlineStr">
         <is>
-          <t>T12 id=14 number=52014</t>
+          <t>T01·T11 4건. T12·T15 없음</t>
         </is>
       </c>
     </row>
     <row r="19" ht="48" customHeight="1">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>E-F03-B03</t>
+          <t>E-F03-B02</t>
         </is>
       </c>
       <c r="B19" s="10" t="n">
@@ -2088,7 +2084,7 @@
       </c>
       <c r="D19" s="3" t="inlineStr">
         <is>
-          <t>T15 대조 삭제 전</t>
+          <t>T12 삭제 전 마커</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
@@ -2098,25 +2094,25 @@
       </c>
       <c r="F19" s="3" t="inlineStr">
         <is>
-          <t>C:\JY-Lab\private-evidence\before\E-F03-B03-T15-control.png</t>
+          <t>C:\JY-Lab\private-evidence\before\E-F03-B02-T12-marker.png</t>
         </is>
       </c>
       <c r="G19" s="3" t="n"/>
       <c r="H19" s="3" t="inlineStr">
         <is>
-          <t>3BA3ED20A657A2AC4CB8336F3474531F7F997301E7DDFC9765A01FC75CA14C3C</t>
+          <t>E6B1424A80D6A20581D38278D80D12CBCA3225DB4B9AC67A61526582624B9B46</t>
         </is>
       </c>
       <c r="I19" s="3" t="inlineStr">
         <is>
-          <t>T15 id=17 number=52017</t>
+          <t>T12 id=14 number=52014</t>
         </is>
       </c>
     </row>
     <row r="20" ht="48" customHeight="1">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>E-F03-A01</t>
+          <t>E-F03-B03</t>
         </is>
       </c>
       <c r="B20" s="10" t="n">
@@ -2129,7 +2125,7 @@
       </c>
       <c r="D20" s="3" t="inlineStr">
         <is>
-          <t>T12 삭제 후 잔존</t>
+          <t>T15 대조 삭제 전</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
@@ -2139,25 +2135,25 @@
       </c>
       <c r="F20" s="3" t="inlineStr">
         <is>
-          <t>C:\JY-Lab\private-evidence\after\E-F03-A01-T12-residual.png</t>
+          <t>C:\JY-Lab\private-evidence\before\E-F03-B03-T15-control.png</t>
         </is>
       </c>
       <c r="G20" s="3" t="n"/>
       <c r="H20" s="3" t="inlineStr">
         <is>
-          <t>0C878A3FBCDEA9D5D7DD5EA3E1A3B3964E5040CFCE49F4460F976EAB10ECDD23</t>
+          <t>3BA3ED20A657A2AC4CB8336F3474531F7F997301E7DDFC9765A01FC75CA14C3C</t>
         </is>
       </c>
       <c r="I20" s="3" t="inlineStr">
         <is>
-          <t>C01 삭제 후 마커 잔존</t>
+          <t>T15 id=17 number=52017</t>
         </is>
       </c>
     </row>
     <row r="21" ht="48" customHeight="1">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>E-F03-A02</t>
+          <t>E-F03-A01</t>
         </is>
       </c>
       <c r="B21" s="10" t="n">
@@ -2170,7 +2166,7 @@
       </c>
       <c r="D21" s="3" t="inlineStr">
         <is>
-          <t>T15 삭제 후 보존</t>
+          <t>T12 삭제 후 잔존</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
@@ -2180,18 +2176,96 @@
       </c>
       <c r="F21" s="3" t="inlineStr">
         <is>
-          <t>C:\JY-Lab\private-evidence\after\E-F03-A02-T15-preserved.png</t>
+          <t>C:\JY-Lab\private-evidence\after\E-F03-A01-T12-residual.png</t>
         </is>
       </c>
       <c r="G21" s="3" t="n"/>
       <c r="H21" s="3" t="inlineStr">
         <is>
+          <t>0C878A3FBCDEA9D5D7DD5EA3E1A3B3964E5040CFCE49F4460F976EAB10ECDD23</t>
+        </is>
+      </c>
+      <c r="I21" s="3" t="inlineStr">
+        <is>
+          <t>C01 삭제 후 마커 잔존</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="48" customHeight="1">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>E-F03-A02</t>
+        </is>
+      </c>
+      <c r="B22" s="10" t="n">
+        <v>46301</v>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>수행자</t>
+        </is>
+      </c>
+      <c r="D22" s="3" t="inlineStr">
+        <is>
+          <t>T15 삭제 후 보존</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>화면</t>
+        </is>
+      </c>
+      <c r="F22" s="3" t="inlineStr">
+        <is>
+          <t>C:\JY-Lab\private-evidence\after\E-F03-A02-T15-preserved.png</t>
+        </is>
+      </c>
+      <c r="G22" s="3" t="n"/>
+      <c r="H22" s="3" t="inlineStr">
+        <is>
           <t>5B576280C64B3E30B77034CBE4A37E40DDBB166FBFF2BEAF33FDE7DC3708A553</t>
         </is>
       </c>
-      <c r="I21" s="3" t="inlineStr">
+      <c r="I22" s="3" t="inlineStr">
         <is>
           <t>대조 티켓 보존</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="48" customHeight="1">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>E-D03-A01</t>
+        </is>
+      </c>
+      <c r="B23" s="10" t="n">
+        <v>46302</v>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>수행자</t>
+        </is>
+      </c>
+      <c r="D23" s="3" t="inlineStr">
+        <is>
+          <t>T12 jy-doc02 로컬 사본</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>파일</t>
+        </is>
+      </c>
+      <c r="F23" s="3" t="inlineStr">
+        <is>
+          <t>C:\JY-Lab\private-evidence\after\jy-doc02-copy.txt</t>
+        </is>
+      </c>
+      <c r="G23" s="3" t="n"/>
+      <c r="H23" s="3" t="n"/>
+      <c r="I23" s="3" t="inlineStr">
+        <is>
+          <t>C01 삭제 후 다운로드. 2026-10-07 09:34, 44바이트. Git 제외. SHA256은 로컬 Get-FileHash</t>
         </is>
       </c>
     </row>
@@ -2347,7 +2421,7 @@
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>PC 다운로드 폴더</t>
+          <t>C:\JY-Lab\private-evidence\after\jy-doc02-copy.txt</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
@@ -2367,7 +2441,7 @@
       </c>
       <c r="G4" s="3" t="inlineStr">
         <is>
-          <t>13장에서 확인</t>
+          <t>2026-10-07 T12에서 다운로드 확인. C01 삭제 후에도 사본 잔존.</t>
         </is>
       </c>
     </row>
@@ -3808,7 +3882,7 @@
       </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
-          <t>종료일(2026-09-14) 이후에도 Active=TRUE·에이전트. 비활성 후 로그인 차단 확인.</t>
+          <t>종료일(2026-09-14) 이후에도 Active=TRUE·에이전트. 비활성 후 새 로그인 차단 확인. users-diff는 S05 active True→False만 변경.</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
@@ -3818,12 +3892,12 @@
       </c>
       <c r="G11" s="3" t="inlineStr">
         <is>
-          <t>E-F01-B01, E-F01-A01</t>
+          <t>E-F01-B01, E-F01-A01, JSON-F01-DIFF</t>
         </is>
       </c>
       <c r="H11" s="3" t="inlineStr">
         <is>
-          <t>재점검은 Retest R-01. 복원·감사로그는 미확인.</t>
+          <t>재점검은 Retest R-01. Sessions 기존 세션 회수·복원·감사로그는 미확인.</t>
         </is>
       </c>
     </row>
@@ -3907,7 +3981,7 @@
       </c>
       <c r="H13" s="3" t="inlineStr">
         <is>
-          <t>재점검은 Retest R-02b. 백업·사본은 미확인.</t>
+          <t>재점검은 Retest R-02b. 사본은 D03. 백업은 미확인.</t>
         </is>
       </c>
     </row>
@@ -4018,18 +4092,22 @@
       </c>
       <c r="E16" s="3" t="inlineStr">
         <is>
-          <t>jy-doc02 등 다운로드 사본의 PC 위치·파기는 화면 미실측.</t>
+          <t>C01 삭제·권한 회수 후에도 T12에서 받은 jy-doc02.txt가 PC에 남음. 2026-10-07 09:34, 44바이트.</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>미확인</t>
-        </is>
-      </c>
-      <c r="G16" s="3" t="n"/>
+          <t>미흡</t>
+        </is>
+      </c>
+      <c r="G16" s="3" t="inlineStr">
+        <is>
+          <t>E-D03-A01</t>
+        </is>
+      </c>
       <c r="H16" s="3" t="inlineStr">
         <is>
-          <t>권한 회수·사용자 삭제로 로컬 사본은 지워지지 않음.</t>
+          <t>USB·DLP 미실시. samples 원본과 별개의 다운로드 사본. T12는 미삭제.</t>
         </is>
       </c>
     </row>
@@ -4178,7 +4256,7 @@
       </c>
       <c r="E20" s="3" t="inlineStr">
         <is>
-          <t>C01 삭제 후 T12(id=14,#52014)에 JY-C01-DELETE-MARKER-ALPHA 잔존. T15(id=17,#52017,jy-doc03.txt)는 보존.</t>
+          <t>C01 삭제 후 T12(id=14,#52014)에 JY-C01-DELETE-MARKER-ALPHA 잔존. T15 보존. 로컬 사본 jy-doc02-copy.txt 잔존.</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
@@ -4193,7 +4271,7 @@
       </c>
       <c r="H20" s="3" t="inlineStr">
         <is>
-          <t>T12는 증적 유지를 위해 삭제하지 않음. 백업·다운로드 사본은 미확인.</t>
+          <t>T12는 증적 유지를 위해 삭제하지 않음. 사본은 E-D03-A01. 백업은 미확인.</t>
         </is>
       </c>
     </row>
@@ -4258,7 +4336,7 @@
       </c>
       <c r="E22" s="3" t="inlineStr">
         <is>
-          <t>F-01~F-03 화면·JSON SHA256 수집. 명부 이메일 .example.test. 토큰 미저장.</t>
+          <t>F-01~F-03 화면·JSON SHA256 수집. users-diff.json은 S05 active True→False만. 명부 이메일 .example.test. 토큰 미저장.</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
@@ -4268,12 +4346,12 @@
       </c>
       <c r="G22" s="3" t="inlineStr">
         <is>
-          <t>Evidence</t>
+          <t>Evidence, JSON-F01-DIFF, E-D03-A01</t>
         </is>
       </c>
       <c r="H22" s="3" t="inlineStr">
         <is>
-          <t>ENV-01 등 환경 증적 해시는 미기입. 원본은 Git 밖.</t>
+          <t>ENV-01·E-D03-A01·JSON-F01-DIFF 해시는 로컬 Get-FileHash 후 기입. 원본은 Git 밖.</t>
         </is>
       </c>
     </row>
@@ -4380,7 +4458,7 @@
       </c>
       <c r="E25" s="3" t="inlineStr">
         <is>
-          <t>F-01·F-02 재점검 적합. F-03은 삭제 범위 적합·참조 잔존 미흡. 잔존 파기는 예정.</t>
+          <t>F-01·F-02 재점검 적합. F-03은 삭제 범위 적합·T12 참조·로컬 사본(D03) 잔존 미흡. 잔존 파기는 예정.</t>
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr">
@@ -4390,7 +4468,7 @@
       </c>
       <c r="G25" s="3" t="inlineStr">
         <is>
-          <t>R-01, R-02a, R-02b, R-03</t>
+          <t>R-01, R-02a, R-02b, R-03, E-D03-A01</t>
         </is>
       </c>
       <c r="H25" s="3" t="inlineStr">
@@ -4621,12 +4699,12 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>E03</t>
+          <t>E03, D03</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>C01 Data Privacy 실행 후 T01·T11은 삭제됐으나 T12(C02, #52014)에 JY-C01-DELETE-MARKER-ALPHA가 남음. T15(C10)는 보존.</t>
+          <t>C01 Data Privacy 실행 후 T01·T11은 삭제됐으나 T12(C02, #52014)에 JY-C01-DELETE-MARKER-ALPHA가 남음. T15(C10)는 보존. 로컬 사본 jy-doc02-copy.txt도 잔존.</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
@@ -4636,7 +4714,7 @@
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>삭제 요청 정보가 다른 고객 티켓에 잔존.</t>
+          <t>삭제 요청 정보가 다른 고객 티켓·PC 다운로드 사본에 잔존.</t>
         </is>
       </c>
       <c r="F5" s="2" t="n">
@@ -4649,7 +4727,7 @@
       </c>
       <c r="H5" s="3" t="inlineStr">
         <is>
-          <t>E-F03-B01, E-F03-B02, E-F03-A01, E-F03-A02</t>
+          <t>E-F03-B01, E-F03-B02, E-F03-A01, E-F03-A02, E-D03-A01</t>
         </is>
       </c>
     </row>
@@ -4858,7 +4936,7 @@
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>T12 잔존 표식·T15 보존을 확인. T12는 증적 유지를 위해 삭제하지 않음.</t>
+          <t>T12 잔존 표식·T15 보존·로컬 jy-doc02-copy.txt(2026-10-07, 44바이트) 잔존을 확인. T12는 증적 유지를 위해 삭제하지 않음.</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">

</xml_diff>

<commit_message>
Add chapter 14 risk, change-request, and exception records.
</commit_message>
<xml_diff>
--- a/reports/JY-Audit-Workbook.xlsx
+++ b/reports/JY-Audit-Workbook.xlsx
@@ -4826,7 +4826,7 @@
       </c>
       <c r="E2" s="3" t="inlineStr">
         <is>
-          <t>수행자</t>
+          <t>시스템 관리자(S01)</t>
         </is>
       </c>
       <c r="F2" s="10" t="n">
@@ -4866,7 +4866,7 @@
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>수행자</t>
+          <t>시스템 관리자(S01)</t>
         </is>
       </c>
       <c r="F3" s="10" t="n">
@@ -4906,7 +4906,7 @@
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>수행자</t>
+          <t>시스템 관리자(S01)</t>
         </is>
       </c>
       <c r="F4" s="10" t="n">
@@ -4946,7 +4946,7 @@
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>수행자</t>
+          <t>개인정보 보호 담당(S02)</t>
         </is>
       </c>
       <c r="F5" s="10" t="n">

</xml_diff>

<commit_message>
docs: record privacy-policy guide type and edition
</commit_message>
<xml_diff>
--- a/reports/JY-Audit-Workbook.xlsx
+++ b/reports/JY-Audit-Workbook.xlsx
@@ -134,7 +134,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<x:sst xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="696" uniqueCount="530">
+<x:sst xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="700" uniqueCount="534">
   <x:si>
     <x:t>C:\JY-Lab\private-evidence\after\E-F03-A02-T15-preserved.png</x:t>
   </x:si>
@@ -1724,6 +1724,18 @@
   </x:si>
   <x:si>
     <x:t>직접 기술 범위 아님</x:t>
+  </x:si>
+  <x:si>
+    <x:t>문서유형</x:t>
+  </x:si>
+  <x:si>
+    <x:t>개정판</x:t>
+  </x:si>
+  <x:si>
+    <x:t>작성지침</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2026.4. 개정</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -2289,9 +2301,9 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="SourcesTable" displayName="SourcesTable" ref="A1:I5" totalsRowBorderDxfId="5">
-  <x:autoFilter ref="A1:I5"/>
-  <x:tableColumns count="9">
+<x:table xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="SourcesTable" displayName="SourcesTable" ref="A1:K8" totalsRowBorderDxfId="5">
+  <x:autoFilter ref="A1:K8"/>
+  <x:tableColumns count="11">
     <x:tableColumn id="1" name="출처ID" dataDxfId="6"/>
     <x:tableColumn id="2" name="기관" dataDxfId="6"/>
     <x:tableColumn id="3" name="제목" dataDxfId="6"/>
@@ -2301,6 +2313,8 @@
     <x:tableColumn id="7" name="URL" dataDxfId="6"/>
     <x:tableColumn id="8" name="관련조항" dataDxfId="6"/>
     <x:tableColumn id="9" name="상태" dataDxfId="6"/>
+    <x:tableColumn id="10" name="문서유형" dataDxfId="6"/>
+    <x:tableColumn id="11" name="개정판" dataDxfId="6"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
@@ -4119,7 +4133,7 @@
     <x:tabColor rgb="ff0f6c6c"/>
     <x:pageSetUpPr autoPageBreaks="1" fitToPage="1"/>
   </x:sheetPr>
-  <x:dimension ref="A1:I8"/>
+  <x:dimension ref="A1:K8"/>
   <x:sheetFormatPr defaultColWidth="8.796875" defaultRowHeight="16.39999999999999857891"/>
   <x:cols>
     <x:col min="1" max="1" width="10" customWidth="1"/>
@@ -4129,9 +4143,11 @@
     <x:col min="7" max="7" width="52" customWidth="1"/>
     <x:col min="8" max="8" width="42" customWidth="1"/>
     <x:col min="9" max="9" width="10" customWidth="1"/>
+    <x:col min="10" max="10" width="14" customWidth="1"/>
+    <x:col min="11" max="11" width="16" customWidth="1"/>
   </x:cols>
   <x:sheetData>
-    <x:row r="1" spans="1:9" ht="28" customHeight="1">
+    <x:row r="1" spans="1:11" ht="28" customHeight="1">
       <x:c r="A1" s="1" t="s">
         <x:v>233</x:v>
       </x:c>
@@ -4159,8 +4175,14 @@
       <x:c r="I1" s="1" t="s">
         <x:v>55</x:v>
       </x:c>
-    </x:row>
-    <x:row r="2" spans="1:9" ht="36" customHeight="1">
+      <x:c r="J1" s="1" t="s">
+        <x:v>530</x:v>
+      </x:c>
+      <x:c r="K1" s="1" t="s">
+        <x:v>531</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" spans="1:11" ht="36" customHeight="1">
       <x:c r="A2" s="2" t="s">
         <x:v>261</x:v>
       </x:c>
@@ -4189,7 +4211,7 @@
         <x:v>48</x:v>
       </x:c>
     </x:row>
-    <x:row r="3" spans="1:9" ht="36" customHeight="1">
+    <x:row r="3" spans="1:11" ht="36" customHeight="1">
       <x:c r="A3" s="2" t="s">
         <x:v>280</x:v>
       </x:c>
@@ -4218,7 +4240,7 @@
         <x:v>48</x:v>
       </x:c>
     </x:row>
-    <x:row r="4" spans="1:9" ht="36" customHeight="1">
+    <x:row r="4" spans="1:11" ht="36" customHeight="1">
       <x:c r="A4" s="2" t="s">
         <x:v>275</x:v>
       </x:c>
@@ -4247,7 +4269,7 @@
         <x:v>48</x:v>
       </x:c>
     </x:row>
-    <x:row r="5" spans="1:9" ht="36" customHeight="1">
+    <x:row r="5" spans="1:11" ht="36" customHeight="1">
       <x:c r="A5" s="2" t="s">
         <x:v>262</x:v>
       </x:c>
@@ -4258,7 +4280,7 @@
         <x:v>195</x:v>
       </x:c>
       <x:c r="D5" s="5">
-        <x:v>46204</x:v>
+        <x:v>46135</x:v>
       </x:c>
       <x:c r="E5" s="7">
         <x:v>46135</x:v>
@@ -4275,8 +4297,14 @@
       <x:c r="I5" s="2" t="s">
         <x:v>48</x:v>
       </x:c>
-    </x:row>
-    <x:row r="6" spans="1:9" ht="36" customHeight="1">
+      <x:c r="J5" s="2" t="s">
+        <x:v>532</x:v>
+      </x:c>
+      <x:c r="K5" s="2" t="s">
+        <x:v>533</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" spans="1:11" ht="36" customHeight="1">
       <x:c r="A6" s="8" t="s">
         <x:v>241</x:v>
       </x:c>
@@ -4287,7 +4315,7 @@
         <x:v>407</x:v>
       </x:c>
       <x:c r="D6" s="5">
-        <x:v>46135</x:v>
+        <x:v>45253</x:v>
       </x:c>
       <x:c r="E6" s="10"/>
       <x:c r="F6" s="10">
@@ -4303,7 +4331,7 @@
         <x:v>11</x:v>
       </x:c>
     </x:row>
-    <x:row r="7" spans="1:9" ht="51.60000000000000142109" customHeight="1">
+    <x:row r="7" spans="1:11" ht="51.60000000000000142109" customHeight="1">
       <x:c r="A7" s="8" t="s">
         <x:v>267</x:v>
       </x:c>
@@ -4330,7 +4358,7 @@
         <x:v>288</x:v>
       </x:c>
     </x:row>
-    <x:row r="8" spans="1:9" s="14" customFormat="1" ht="36" customHeight="1">
+    <x:row r="8" spans="1:11" s="14" customFormat="1" ht="36" customHeight="1">
       <x:c r="A8" s="8" t="s">
         <x:v>401</x:v>
       </x:c>

</xml_diff>

<commit_message>
docs: fill source document type and edition
</commit_message>
<xml_diff>
--- a/reports/JY-Audit-Workbook.xlsx
+++ b/reports/JY-Audit-Workbook.xlsx
@@ -134,7 +134,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<x:sst xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="700" uniqueCount="534">
+<x:sst xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="712" uniqueCount="546">
   <x:si>
     <x:t>C:\JY-Lab\private-evidence\after\E-F03-A02-T15-preserved.png</x:t>
   </x:si>
@@ -1736,6 +1736,42 @@
   </x:si>
   <x:si>
     <x:t>2026.4. 개정</x:t>
+  </x:si>
+  <x:si>
+    <x:t>법률</x:t>
+  </x:si>
+  <x:si>
+    <x:t>법률 제21445호</x:t>
+  </x:si>
+  <x:si>
+    <x:t>대통령령</x:t>
+  </x:si>
+  <x:si>
+    <x:t>대통령령 제36671호</x:t>
+  </x:si>
+  <x:si>
+    <x:t>고시</x:t>
+  </x:si>
+  <x:si>
+    <x:t>개인정보보호위원회고시 제2026-9호</x:t>
+  </x:si>
+  <x:si>
+    <x:t>인증기준 안내서</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2023.11</x:t>
+  </x:si>
+  <x:si>
+    <x:t>국제표준</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2025 제2판</x:t>
+  </x:si>
+  <x:si>
+    <x:t>기술 상세가이드</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2025-12-24 게시</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -4210,6 +4246,12 @@
       <x:c r="I2" s="2" t="s">
         <x:v>48</x:v>
       </x:c>
+      <x:c r="J2" s="2" t="s">
+        <x:v>534</x:v>
+      </x:c>
+      <x:c r="K2" s="2" t="s">
+        <x:v>535</x:v>
+      </x:c>
     </x:row>
     <x:row r="3" spans="1:11" ht="36" customHeight="1">
       <x:c r="A3" s="2" t="s">
@@ -4239,6 +4281,12 @@
       <x:c r="I3" s="2" t="s">
         <x:v>48</x:v>
       </x:c>
+      <x:c r="J3" s="2" t="s">
+        <x:v>536</x:v>
+      </x:c>
+      <x:c r="K3" s="2" t="s">
+        <x:v>537</x:v>
+      </x:c>
     </x:row>
     <x:row r="4" spans="1:11" ht="36" customHeight="1">
       <x:c r="A4" s="2" t="s">
@@ -4268,6 +4316,12 @@
       <x:c r="I4" s="2" t="s">
         <x:v>48</x:v>
       </x:c>
+      <x:c r="J4" s="2" t="s">
+        <x:v>538</x:v>
+      </x:c>
+      <x:c r="K4" s="2" t="s">
+        <x:v>539</x:v>
+      </x:c>
     </x:row>
     <x:row r="5" spans="1:11" ht="36" customHeight="1">
       <x:c r="A5" s="2" t="s">
@@ -4330,6 +4384,12 @@
       <x:c r="I6" s="8" t="s">
         <x:v>11</x:v>
       </x:c>
+      <x:c r="J6" s="8" t="s">
+        <x:v>540</x:v>
+      </x:c>
+      <x:c r="K6" s="8" t="s">
+        <x:v>541</x:v>
+      </x:c>
     </x:row>
     <x:row r="7" spans="1:11" ht="51.60000000000000142109" customHeight="1">
       <x:c r="A7" s="8" t="s">
@@ -4357,6 +4417,12 @@
       <x:c r="I7" s="8" t="s">
         <x:v>288</x:v>
       </x:c>
+      <x:c r="J7" s="8" t="s">
+        <x:v>542</x:v>
+      </x:c>
+      <x:c r="K7" s="8" t="s">
+        <x:v>543</x:v>
+      </x:c>
     </x:row>
     <x:row r="8" spans="1:11" s="14" customFormat="1" ht="36" customHeight="1">
       <x:c r="A8" s="8" t="s">
@@ -4383,6 +4449,12 @@
       </x:c>
       <x:c r="I8" s="8" t="s">
         <x:v>529</x:v>
+      </x:c>
+      <x:c r="J8" s="8" t="s">
+        <x:v>544</x:v>
+      </x:c>
+      <x:c r="K8" s="8" t="s">
+        <x:v>545</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
docs: count initial checks and fix evidence links
</commit_message>
<xml_diff>
--- a/reports/JY-Audit-Workbook.xlsx
+++ b/reports/JY-Audit-Workbook.xlsx
@@ -4791,7 +4791,7 @@
         <x:v>41</x:v>
       </x:c>
       <x:c r="I2" s="3" t="s">
-        <x:v>44</x:v>
+        <x:v>479</x:v>
       </x:c>
     </x:row>
     <x:row r="3" spans="1:9" ht="36" customHeight="1">
@@ -4818,7 +4818,7 @@
         <x:v>41</x:v>
       </x:c>
       <x:c r="I3" s="3" t="s">
-        <x:v>50</x:v>
+        <x:v>479</x:v>
       </x:c>
     </x:row>
     <x:row r="4" spans="1:9" ht="36" customHeight="1">
@@ -4845,7 +4845,7 @@
         <x:v>41</x:v>
       </x:c>
       <x:c r="I4" s="3" t="s">
-        <x:v>21</x:v>
+        <x:v>479</x:v>
       </x:c>
     </x:row>
     <x:row r="5" spans="1:9" ht="36" customHeight="1">
@@ -5376,7 +5376,7 @@
     <x:tabColor rgb="ff8a5a12"/>
     <x:pageSetUpPr autoPageBreaks="1" fitToPage="1"/>
   </x:sheetPr>
-  <x:dimension ref="A1:H25"/>
+  <x:dimension ref="A1:K25"/>
   <x:sheetFormatPr defaultColWidth="8.796875" defaultRowHeight="16.39999999999999857891"/>
   <x:cols>
     <x:col min="1" max="2" width="10" customWidth="1"/>
@@ -5385,9 +5385,11 @@
     <x:col min="6" max="6" width="10" customWidth="1"/>
     <x:col min="7" max="7" width="23" customWidth="1"/>
     <x:col min="8" max="8" width="28" customWidth="1"/>
+    <x:col min="10" max="10" width="18" customWidth="1"/>
+    <x:col min="11" max="11" width="16" customWidth="1"/>
   </x:cols>
   <x:sheetData>
-    <x:row r="1" spans="1:8" ht="28" customHeight="1">
+    <x:row r="1" spans="1:11" ht="28" customHeight="1">
       <x:c r="A1" s="1" t="s">
         <x:v>275</x:v>
       </x:c>
@@ -5412,8 +5414,18 @@
       <x:c r="H1" s="1" t="s">
         <x:v>501</x:v>
       </x:c>
-    </x:row>
-    <x:row r="2" spans="1:8" ht="48" customHeight="1">
+      <x:c r="J1" t="inlineStr">
+        <x:is>
+          <x:t>초기 판정 집계</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K1" t="inlineStr">
+        <x:is>
+          <x:t>2026-10-15</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="2" spans="1:11" ht="48" customHeight="1">
       <x:c r="A2" s="2" t="s">
         <x:v>451</x:v>
       </x:c>
@@ -5438,8 +5450,17 @@
       <x:c r="H2" s="3" t="s">
         <x:v>574</x:v>
       </x:c>
-    </x:row>
-    <x:row r="3" spans="1:8" ht="48" customHeight="1">
+      <x:c r="J2" t="inlineStr">
+        <x:is>
+          <x:t>적합</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K2">
+        <x:f>COUNTIF(F$2:F$25,"적합")</x:f>
+        <x:v>8</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" spans="1:11" ht="48" customHeight="1">
       <x:c r="A3" s="2" t="s">
         <x:v>483</x:v>
       </x:c>
@@ -5464,8 +5485,17 @@
       <x:c r="H3" s="3" t="s">
         <x:v>531</x:v>
       </x:c>
-    </x:row>
-    <x:row r="4" spans="1:8" ht="48" customHeight="1">
+      <x:c r="J3" t="inlineStr">
+        <x:is>
+          <x:t>미흡</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K3">
+        <x:f>COUNTIF(F$2:F$25,"미흡")</x:f>
+        <x:v>13</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" spans="1:11" ht="48" customHeight="1">
       <x:c r="A4" s="2" t="s">
         <x:v>497</x:v>
       </x:c>
@@ -5490,8 +5520,17 @@
       <x:c r="H4" s="3" t="s">
         <x:v>131</x:v>
       </x:c>
-    </x:row>
-    <x:row r="5" spans="1:8" ht="48" customHeight="1">
+      <x:c r="J4" t="inlineStr">
+        <x:is>
+          <x:t>미확인</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K4">
+        <x:f>COUNTIF(F$2:F$25,"미확인")</x:f>
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" spans="1:11" ht="48" customHeight="1">
       <x:c r="A5" s="2" t="s">
         <x:v>492</x:v>
       </x:c>
@@ -5516,8 +5555,17 @@
       <x:c r="H5" s="3" t="s">
         <x:v>576</x:v>
       </x:c>
-    </x:row>
-    <x:row r="6" spans="1:8" ht="48" customHeight="1">
+      <x:c r="J5" t="inlineStr">
+        <x:is>
+          <x:t>적용 제외</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K5">
+        <x:f>COUNTIF(F$2:F$25,"적용 제외")</x:f>
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" spans="1:11" ht="48" customHeight="1">
       <x:c r="A6" s="2" t="s">
         <x:v>468</x:v>
       </x:c>
@@ -5541,6 +5589,15 @@
       </x:c>
       <x:c r="H6" s="3" t="s">
         <x:v>549</x:v>
+      </x:c>
+      <x:c r="J6" t="inlineStr">
+        <x:is>
+          <x:t>합계</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K6">
+        <x:f>K2+K3+K4+K5</x:f>
+        <x:v>24</x:v>
       </x:c>
     </x:row>
     <x:row r="7" spans="1:8" ht="48" customHeight="1">
@@ -5873,7 +5930,7 @@
         <x:v>486</x:v>
       </x:c>
       <x:c r="G19" s="3" t="s">
-        <x:v>555</x:v>
+        <x:v>78</x:v>
       </x:c>
       <x:c r="H19" s="3" t="s">
         <x:v>517</x:v>

</xml_diff>

<commit_message>
docs: add final review sheet
</commit_message>
<xml_diff>
--- a/reports/JY-Audit-Workbook.xlsx
+++ b/reports/JY-Audit-Workbook.xlsx
@@ -23,6 +23,8 @@
     <x:sheet name="Actions" sheetId="9" r:id="rId12"/>
     <x:sheet name="Retest" sheetId="10" r:id="rId13"/>
     <x:sheet name="Evidence" sheetId="11" r:id="rId14"/>
+    <x:sheet name="Incident" sheetId="12" r:id="rId15"/>
+    <x:sheet name="FinalReview" sheetId="13" r:id="rId16"/>
   </x:sheets>
   <x:definedNames>
     <x:definedName name="_xlnm.Print_Titles" localSheetId="0">Scope!$1:$1</x:definedName>
@@ -36,6 +38,8 @@
     <x:definedName name="_xlnm.Print_Titles" localSheetId="8">Actions!$1:$1</x:definedName>
     <x:definedName name="_xlnm.Print_Titles" localSheetId="9">'Retest'!$1:$1</x:definedName>
     <x:definedName name="_xlnm.Print_Titles" localSheetId="10">Evidence!$1:$1</x:definedName>
+    <x:definedName name="_xlnm.Print_Titles" localSheetId="11">Incident!$1:$1</x:definedName>
+    <x:definedName name="_xlnm.Print_Titles" localSheetId="12">FinalReview!$1:$1</x:definedName>
   </x:definedNames>
   <x:calcPr xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:hs="http://schemas.haansoft.com/office/spreadsheet/8.0" mc:Ignorable="hs" hs:hclCalcId="904"/>
 </x:workbook>
@@ -2658,6 +2662,26 @@
 </x:table>
 </file>
 
+<file path=xl/tables/table12.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="12" name="FinalReviewTable" displayName="FinalReviewTable" ref="A1:K25" totalsRowBorderDxfId="5">
+  <x:autoFilter ref="A1:K25"/>
+  <x:tableColumns count="11">
+    <x:tableColumn id="1" name="항목ID" dataDxfId="9"/>
+    <x:tableColumn id="2" name="검토대상" dataDxfId="9"/>
+    <x:tableColumn id="3" name="초기판정" dataDxfId="9"/>
+    <x:tableColumn id="4" name="현재관측" dataDxfId="9"/>
+    <x:tableColumn id="5" name="현재상태" dataDxfId="9"/>
+    <x:tableColumn id="6" name="근거" dataDxfId="9"/>
+    <x:tableColumn id="7" name="한계" dataDxfId="9"/>
+    <x:tableColumn id="8" name="담당" dataDxfId="9"/>
+    <x:tableColumn id="9" name="기한" dataDxfId="9"/>
+    <x:tableColumn id="10" name="검토일" dataDxfId="9"/>
+    <x:tableColumn id="11" name="인계결정" dataDxfId="9"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
+</file>
+
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
 <x:table xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="AssetsTable" displayName="AssetsTable" ref="A1:G5" totalsRowBorderDxfId="5">
   <x:autoFilter ref="A1:G5"/>
@@ -4446,6 +4470,1563 @@
 </x:worksheet>
 </file>
 
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetPr codeName="Sheet12">
+    <x:tabColor rgb="ff1f4e79"/>
+    <x:pageSetUpPr autoPageBreaks="1" fitToPage="1"/>
+  </x:sheetPr>
+  <x:dimension ref="A1:L3"/>
+  <x:sheetFormatPr defaultRowHeight="18"/>
+  <x:cols>
+    <x:col min="1" max="10" width="18" customWidth="1"/>
+    <x:col min="12" max="12" width="28" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" spans="1:12" ht="28" customHeight="1">
+      <x:c r="A1" s="1" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">훈련ID</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B1" s="1" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">시점종류</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C1" s="1" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">모의시각/실제기록일</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D1" s="1" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">상황정보</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E1" s="1" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">역할</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F1" s="1" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">판단</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G1" s="1" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">조치</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H1" s="1" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">근거</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I1" s="1" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">미확인</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J1" s="1" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">개선과제</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="L1" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">기준일</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="2" spans="12:12">
+      <x:c r="L2" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">2026-10-15</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="3" spans="12:12">
+      <x:c r="L3" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">본문은 11단계에서 채운다.</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:autoFilter ref="A1:J1"/>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetPr codeName="Sheet13">
+    <x:tabColor rgb="ff1e4d3a"/>
+    <x:pageSetUpPr autoPageBreaks="1" fitToPage="1"/>
+  </x:sheetPr>
+  <x:dimension ref="A1:M25"/>
+  <x:sheetFormatPr defaultRowHeight="18"/>
+  <x:cols>
+    <x:col min="1" max="1" width="12" customWidth="1"/>
+    <x:col min="2" max="2" width="14" customWidth="1"/>
+    <x:col min="3" max="3" width="14" customWidth="1"/>
+    <x:col min="4" max="7" width="36" customWidth="1"/>
+    <x:col min="8" max="8" width="24" customWidth="1"/>
+    <x:col min="9" max="10" width="14" customWidth="1"/>
+    <x:col min="11" max="11" width="32" customWidth="1"/>
+    <x:col min="13" max="13" width="42" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" spans="1:13" ht="28" customHeight="1">
+      <x:c r="A1" s="1" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">항목ID</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B1" s="1" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">검토대상</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C1" s="1" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">초기판정</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D1" s="1" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">현재관측</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E1" s="1" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">현재상태</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F1" s="1" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">근거</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G1" s="1" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">한계</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H1" s="1" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">담당</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I1" s="1" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">기한</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J1" s="1" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">검토일</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K1" s="1" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">인계결정</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="M1" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">기준일</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="2" spans="1:13" ht="48" customHeight="1">
+      <x:c r="A2" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">A01</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B2" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">범위</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C2" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">적합</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D2" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">2026-10-15에 scope 문서를 다시 열지 않음.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E2" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">초기 판정 유지</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F2" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">docs/scope.md.txt</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G2" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">모의와 실제 구별. 범위 문서 기준.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H2" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">미정</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I2" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">미정</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J2" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">2026-10-15</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K2" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">초기 적합 유지</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="M2" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">2026-10-15</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="3" spans="1:13" ht="48" customHeight="1">
+      <x:c r="A3" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">A02</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B3" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">법령버전</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C3" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">적합</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D3" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">2026-10-14에 법령 3개 머리글과 ISMS-P 쪽수를 확인. 조문 본문은 다시 읽지 않음.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E3" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">초기 판정 유지</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F3" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">S-L01~S-L05. S-L04 시행일은 비움.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G3" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">머리글 확인이며 조문 재독은 아님. S-L06과 S-L07은 재확인하지 않음.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H3" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">미정</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I3" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">미정</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J3" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">2026-10-14</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K3" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">초기 적합 유지</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="M3" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">초기 집계는 Checks에만 둔다. 이 시트와 합산하지 않음.</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="4" spans="1:11" ht="48" customHeight="1">
+      <x:c r="A4" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">A03</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B4" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">흐름</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C4" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">적합</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D4" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">docs/data-flow.pdf 해시를 2026-10-14에 처음 기록.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E4" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">초기 판정 유지</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F4" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">DF-01</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G4" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">논리흐름. 백업 실측 아님.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H4" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">미정</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I4" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">미정</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J4" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">2026-10-14</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K4" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">초기 적합 유지</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="5" spans="1:11" ht="48" customHeight="1">
+      <x:c r="A5" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">A04</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B5" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">책임</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C5" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">적합</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D5" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">2026-10-15에 인터뷰 문서를 다시 열지 않음.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E5" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">초기 판정 유지</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F5" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">docs/interview.md.txt</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G5" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">실제 조직 운영과 서명은 미확인.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H5" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">미정</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I5" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">미정</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J5" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">2026-10-15</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K5" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">초기 적합 유지. 실제 서명은 미확인</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="6" spans="1:11" ht="48" customHeight="1">
+      <x:c r="A6" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">B01</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B6" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">목적항목</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C6" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">적합</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D6" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">2026-10-15에 티켓 양식을 다시 열지 않음.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E6" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">초기 판정 유지</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F6" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">tickets.csv, control-notes.md</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G6" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">목적별 세분 고지는 티켓 양식에 없음.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H6" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">미정</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I6" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">미정</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J6" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">2026-10-15</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K6" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">초기 적합 유지</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="7" spans="1:11" ht="48" customHeight="1">
+      <x:c r="A7" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">B02</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B7" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">처리방침</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C7" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">미흡</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D7" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">2026-10-15에 방침 문서를 다시 열지 않음.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E7" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">초기 미흡 유지</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F7" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">02-privacy-policy.md.txt</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G7" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">운영과 방침 문구가 다를 수 있음.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H7" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">미정</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I7" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">미정</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J7" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">2026-10-15</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K7" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">미흡 유지. 문안 수정은 이후 단계</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="8" spans="1:11" ht="48" customHeight="1">
+      <x:c r="A8" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">B03</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B8" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">위탁제3자</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C8" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">미흡</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D8" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">2026-10-15에 위탁 문서를 다시 열지 않음.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E8" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">초기 미흡 유지</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F8" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">03-outsourcing.md.txt</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G8" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">연간 수탁 점검은 D01.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H8" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">미정</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I8" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">미정</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J8" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">2026-10-15</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K8" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">미흡 유지</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="9" spans="1:11" ht="48" customHeight="1">
+      <x:c r="A9" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">B04</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B9" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">권리</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C9" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">미확인</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D9" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">권리 메일은 보내지 않음. 모의 절차 문서는 아직 없음.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E9" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">미확인 유지</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F9" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">E-F03-B01</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G9" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">실제 발송 없음. 초기 권리 절차 문서 없음.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H9" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">미정</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I9" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">미정</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J9" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">2026-10-15</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K9" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">미확인 유지. 모의 기록은 11단계</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="10" spans="1:11" ht="48" customHeight="1">
+      <x:c r="A10" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">C01</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B10" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">계정발급</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C10" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">적합</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D10" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">직원 6명의 active 요약은 users-active.csv. 이메일은 공개 요약에 없음.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E10" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">초기 판정 유지</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F10" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Accounts, evidence/sanitized/users-active.csv</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G10" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">가상 명부. S01~S03 증적ID는 Evidence에 없어 미확인.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H10" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">미정</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I10" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">미정</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J10" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">2026-10-15</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K10" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">초기 적합 유지</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="11" spans="1:11" ht="48" customHeight="1">
+      <x:c r="A11" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">C02</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B11" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">종료계정</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C11" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">미흡</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D11" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">S05 active가 true에서 false. 로그인 후 캡처만으로 입력 계정을 독립 식별하기 어려움. 재점검 R-01은 적합.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E11" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">초기 미흡 유지. 재점검 적합과 합산하지 않음</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F11" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">E-F01-B01, E-F01-A01, evidence/sanitized/users-active.csv</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G11" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">기존 세션과 외부 토큰 회수는 미확인. F-01 전 화면은 T02 #52020이고 내부ID는 미확인.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H11" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">시스템 관리자(S01)</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I11" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">2026-10-06</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J11" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">2026-10-15</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K11" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">초기 미흡 유지. A-01 상태는 완료</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="12" spans="1:11" ht="48" customHeight="1">
+      <x:c r="A12" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">C03</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B12" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">최소권한</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C12" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">미흡</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D12" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">S04 권한 없음 화면과 T02 #52003 정상업무 화면을 확인. 재점검 R-02a는 적합. #52003은 F-01의 #52020과 다른 티켓.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E12" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">초기 미흡 유지. 재점검 적합과 합산하지 않음</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F12" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">E-F02-B01, E-F02-A01, E-F02-A02</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G12" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">후 캡처의 T11 주소와 번호, 권한 회수 후 삭제 전 순서 근거가 부족. S06 차단과 S03 제한업무 후 시험은 미확인. 화면의 찾을 수 없음은 과거 권한 회수 증명이 아님.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H12" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">시스템 관리자(S01)</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I12" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">2026-10-06</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J12" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">2026-10-15</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K12" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">초기 미흡 유지. A-02a 상태는 완료</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="13" spans="1:11" ht="48" customHeight="1">
+      <x:c r="A13" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">C04</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B13" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">고객공유</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C13" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">미흡</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D13" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">고객 본인 목록은 유지되고 타인 목록은 비공유. 재점검 R-02b는 적합. 후 목록에는 T02 #52020, #52003과 T12 #52029, #52014가 같이 있음.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E13" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">초기 미흡 유지. 재점검 적합과 합산하지 않음</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F13" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">E-F02-B03, E-F02-A03</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G13" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">직접 T01 URL과 첨부 거부 대상은 식별이 부족. 목록 숨김을 직접 접근 차단으로 보지 않음.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H13" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">시스템 관리자(S01)</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I13" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">2026-10-06</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J13" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">2026-10-15</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K13" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">초기 미흡 유지. A-02b 상태는 완료</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="14" spans="1:11" ht="48" customHeight="1">
+      <x:c r="A14" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">D01</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B14" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">수탁감독</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C14" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">미흡</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D14" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">2026-10-15에 수탁 실적 문서를 다시 열지 않음.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E14" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">초기 미흡 유지</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F14" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">03-outsourcing.md.txt</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G14" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">수탁 감독 실적은 문서상 확인 불가.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H14" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">미정</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I14" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">미정</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J14" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">2026-10-15</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K14" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">미흡 유지</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="15" spans="1:11" ht="48" customHeight="1">
+      <x:c r="A15" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">D02</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B15" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">유지보수</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C15" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">미흡</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D15" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">S06 차단 후 시험은 미확인. E-F02-B02는 공개 제외.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E15" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">초기 미흡 유지</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F15" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">E-F02-B02</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G15" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">필요 시 한시 권한 절차는 문서에 없음.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H15" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">미정</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I15" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">미정</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J15" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">2026-10-15</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K15" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">미흡 유지</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="16" spans="1:11" ht="48" customHeight="1">
+      <x:c r="A16" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">D03</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B16" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">다운로드</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C16" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">미흡</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D16" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">jy-doc02-copy.txt 해시가 2026-10-12와 같음. 사본은 남음.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E16" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">초기 미흡 유지</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F16" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">E-D03-A01</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G16" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">USB와 DLP는 하지 않음. T12는 삭제하지 않음.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H16" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">개인정보 보호 담당(S02)</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I16" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">2026-10-06</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J16" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">2026-10-15</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K16" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">미흡 유지. A-03은 기한 경과/미완료</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="17" spans="1:11" ht="48" customHeight="1">
+      <x:c r="A17" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">D04</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B17" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">교육검토</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C17" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">미흡</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D17" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">2026-10-15에 교육 기록을 만들지 않음.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E17" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">초기 미흡 유지</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F17" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">없음</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G17" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">장기 서명과 이수 증빙 없음.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H17" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">미정</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I17" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">미정</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J17" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">2026-10-15</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K17" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">미흡 유지. 교육 파일은 이후 단계</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="18" spans="1:11" ht="48" customHeight="1">
+      <x:c r="A18" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">E01</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B18" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">보유파기</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C18" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">미흡</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D18" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">2026-10-15에 보유 문서를 다시 열지 않음.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E18" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">초기 미흡 유지</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F18" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">05-retention.md.txt</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G18" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">임의 연수를 적지 않음. 원문 대조만.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H18" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">미정</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I18" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">미정</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J18" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">2026-10-15</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K18" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">미흡 유지</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="19" spans="1:11" ht="48" customHeight="1">
+      <x:c r="A19" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">E02</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B19" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">사용자삭제</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C19" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">적합</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D19" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">미리보기 4건은 T01 #52002, T11 #52013, T01 #52018, T11 #52028. #52018 그룹은 Users. 별칭은 E-F03-B01로 연결.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E19" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">초기 적합 유지. 판정 범위는 미리보기 삭제 범위만</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F19" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">E-F03-B01</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G19" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">완료 화면은 다시 보지 않음. 참조 잔존은 E03.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H19" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">미정</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I19" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">미정</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J19" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">2026-10-15</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K19" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">삭제 범위만 적합. 잔존은 E03</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="20" spans="1:11" ht="48" customHeight="1">
+      <x:c r="A20" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">E03</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B20" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">참조잔존</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C20" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">미흡</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D20" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">T12 #52014에 마커와 첨부가 남음. T15 #52017은 보존. 로컬 사본이 남음. 백업 잔존은 미확인.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E20" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">초기 미흡 유지</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F20" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">E-F03-A01, E-F03-A02, E-D03-A01</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G20" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">삭제 미리보기와 completed 상태를 구분. T12 추가 삭제는 종료 조건이 아님. T15 보존은 시험 대조군.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H20" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">개인정보 보호 담당(S02)</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I20" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">2026-10-06</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J20" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">2026-10-15</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K20" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">미흡 유지. A-03은 기한 경과/미완료. 새 목표일과 다음 검토일은 미정</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="21" spans="1:11" ht="48" customHeight="1">
+      <x:c r="A21" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">E04</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B21" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">백업연계</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C21" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">미확인</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D21" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">백업 복구를 시험하지 않음.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E21" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">미확인 유지</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F21" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">없음</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G21" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">컨테이너 실행은 백업 성공이 아님.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H21" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">미정</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I21" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">미정</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J21" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">2026-10-15</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K21" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">미확인 유지. 백업 확인 전에는 완료로 적지 않음</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="22" spans="1:11" ht="48" customHeight="1">
+      <x:c r="A22" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">F01</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B22" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">증적품질</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C22" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">적합</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D22" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">2026-10-14에 ENV 해시와 data-flow.pdf 해시를 기록. 2026-10-15에 공개 10장과 users-active.csv 해시를 기록.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E22" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">초기 적합 유지. 판정 칸은 바꾸지 않음</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F22" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Evidence</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G22" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">원본 JSON과 PNG는 Git 밖. 공개본은 evidence/sanitized.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H22" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">미정</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I22" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">미정</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J22" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">2026-10-15</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K22" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">초기 적합 유지</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="23" spans="1:11" ht="48" customHeight="1">
+      <x:c r="A23" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">F02</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B23" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">사고대응</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C23" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">미흡</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D23" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">도상훈련 표는 2026-10-15에 채우지 않음. Incident 시트는 제목만 있음.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E23" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">초기 미흡 유지</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F23" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">06-incident.md.txt</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G23" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">실제 신고를 하지 않음. 72시간을 단정하지 않음.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H23" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">미정</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I23" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">미정</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J23" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">2026-10-15</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K23" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">미흡 유지. 훈련 기록은 11단계</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="24" spans="1:11" ht="48" customHeight="1">
+      <x:c r="A24" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">F03</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B24" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">AI검토</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C24" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">적용 제외</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D24" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">외부 AI 요약도구는 연결하지 않음.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E24" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">적용 제외 유지</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F24" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">없음</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G24" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">공격시험을 하지 않음.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H24" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">미정</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I24" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">미정</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J24" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">2026-10-15</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K24" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">적용 제외 유지</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="25" spans="1:11" ht="48" customHeight="1">
+      <x:c r="A25" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">F04</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B25" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">이행재점검</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C25" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">미흡</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D25" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">R-01, R-02a, R-02b는 적합이고 R-03은 미흡. 초기 Checks 미흡을 적합으로 덮지 않음.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E25" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">초기 미흡 유지. 재점검 적합 3건과 합산하지 않음</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F25" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">R-01, R-02a, R-02b, R-03</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G25" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">F-03 잔존을 완료로 올리지 않음. E04 백업은 미확인.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H25" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">개인정보 보호 담당(S02)</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I25" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">2026-10-06</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J25" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">2026-10-15</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K25" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">미흡 유지. A-03은 기한 경과/미완료</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:tableParts count="1">
+    <x:tablePart r:id="rId1"/>
+  </x:tableParts>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetPr codeName="Sheet2">

</xml_diff>

<commit_message>
docs: add current risk scores to findings
</commit_message>
<xml_diff>
--- a/reports/JY-Audit-Workbook.xlsx
+++ b/reports/JY-Audit-Workbook.xlsx
@@ -2787,9 +2787,9 @@
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="8" name="FindingsTable" displayName="FindingsTable" ref="A1:H5" totalsRowBorderDxfId="5">
-  <x:autoFilter ref="A1:H5"/>
-  <x:tableColumns count="8">
+<x:table xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="8" name="FindingsTable" displayName="FindingsTable" ref="A1:R5" totalsRowBorderDxfId="5">
+  <x:autoFilter ref="A1:R5"/>
+  <x:tableColumns count="18">
     <x:tableColumn id="1" name="발견ID" dataDxfId="9"/>
     <x:tableColumn id="2" name="연결점검" dataDxfId="9"/>
     <x:tableColumn id="3" name="사실" dataDxfId="9"/>
@@ -2798,6 +2798,16 @@
     <x:tableColumn id="6" name="위험점수" dataDxfId="9"/>
     <x:tableColumn id="7" name="우선순위" dataDxfId="9"/>
     <x:tableColumn id="8" name="근거" dataDxfId="9"/>
+    <x:tableColumn id="9" name="최종가능성" dataDxfId="9"/>
+    <x:tableColumn id="10" name="최종영향" dataDxfId="9"/>
+    <x:tableColumn id="11" name="최종점수" dataDxfId="9"/>
+    <x:tableColumn id="12" name="최종우선순위" dataDxfId="9"/>
+    <x:tableColumn id="13" name="산정근거" dataDxfId="9"/>
+    <x:tableColumn id="14" name="평가기준일" dataDxfId="9"/>
+    <x:tableColumn id="15" name="잔여가능성" dataDxfId="9"/>
+    <x:tableColumn id="16" name="잔여영향" dataDxfId="9"/>
+    <x:tableColumn id="17" name="잔여점수" dataDxfId="9"/>
+    <x:tableColumn id="18" name="잔여우선순위" dataDxfId="9"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
@@ -7708,7 +7718,7 @@
     <x:tabColor rgb="ff7b241c"/>
     <x:pageSetUpPr autoPageBreaks="1" fitToPage="1"/>
   </x:sheetPr>
-  <x:dimension ref="A1:H5"/>
+  <x:dimension ref="A1:R5"/>
   <x:sheetFormatPr defaultColWidth="8.796875" defaultRowHeight="16.39999999999999857891"/>
   <x:cols>
     <x:col min="1" max="2" width="10" customWidth="1"/>
@@ -7716,9 +7726,14 @@
     <x:col min="4" max="4" width="32" customWidth="1"/>
     <x:col min="5" max="7" width="10" customWidth="1"/>
     <x:col min="8" max="8" width="28" customWidth="1"/>
+    <x:col min="9" max="12" width="14" customWidth="1"/>
+    <x:col min="13" max="13" width="42" customWidth="1"/>
+    <x:col min="14" max="14" width="14" customWidth="1"/>
+    <x:col min="15" max="16" width="14" customWidth="1"/>
+    <x:col min="17" max="18" width="14" customWidth="1"/>
   </x:cols>
   <x:sheetData>
-    <x:row r="1" spans="1:8" ht="28" customHeight="1">
+    <x:row r="1" spans="1:18" ht="28" customHeight="1">
       <x:c r="A1" s="1" t="s">
         <x:v>363</x:v>
       </x:c>
@@ -7743,8 +7758,58 @@
       <x:c r="H1" s="1" t="s">
         <x:v>469</x:v>
       </x:c>
-    </x:row>
-    <x:row r="2" spans="1:8" ht="48" customHeight="1">
+      <x:c r="I1" s="1" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">최종가능성</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J1" s="1" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">최종영향</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K1" s="1" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">최종점수</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="L1" s="1" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">최종우선순위</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="M1" s="1" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">산정근거</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="N1" s="1" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">평가기준일</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="O1" s="1" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">잔여가능성</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="P1" s="1" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">잔여영향</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="Q1" s="1" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">잔여점수</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="R1" s="1" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">잔여우선순위</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="2" spans="1:18" ht="48" customHeight="1">
       <x:c r="A2" s="2" t="s">
         <x:v>315</x:v>
       </x:c>
@@ -7769,8 +7834,51 @@
       <x:c r="H2" s="3" t="s">
         <x:v>520</x:v>
       </x:c>
-    </x:row>
-    <x:row r="3" spans="1:8" ht="48" customHeight="1">
+      <x:c r="I2" s="2">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="J2" s="2">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="K2" s="2">
+        <x:f>I2*J2</x:f>
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="L2" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">계획</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="M2" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">종료 뒤 T02 #52020 열람. 내부ID는 미확인. #52003은 다른 티켓. 영향은 일부 고객 상담.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="N2" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">2026-10-15</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="O2" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">미확인</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="P2" s="2">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="Q2" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">미확인</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="R2" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">미확인</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="3" spans="1:18" ht="48" customHeight="1">
       <x:c r="A3" s="2" t="s">
         <x:v>287</x:v>
       </x:c>
@@ -7795,8 +7903,51 @@
       <x:c r="H3" s="3" t="s">
         <x:v>554</x:v>
       </x:c>
-    </x:row>
-    <x:row r="4" spans="1:8" ht="48" customHeight="1">
+      <x:c r="I3" s="2">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="J3" s="2">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="K3" s="2">
+        <x:f>I3*J3</x:f>
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="L3" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">계획</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="M3" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">T11 #52028 열람. 일부 고객 상담. Restricted 이름만으로 영향 3을 주지 않음.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="N3" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">2026-10-15</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="O3" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">미확인</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="P3" s="2">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="Q3" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">미확인</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="R3" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">미확인</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="4" spans="1:18" ht="48" customHeight="1">
       <x:c r="A4" s="2" t="s">
         <x:v>381</x:v>
       </x:c>
@@ -7821,8 +7972,51 @@
       <x:c r="H4" s="3" t="s">
         <x:v>66</x:v>
       </x:c>
-    </x:row>
-    <x:row r="5" spans="1:8" ht="48" customHeight="1">
+      <x:c r="I4" s="2">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="J4" s="2">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="K4" s="2">
+        <x:f>I4*J4</x:f>
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="L4" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">계획</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="M4" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">C02가 조직 목록에서 T01을 열람. 일부 고객 상담.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="N4" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">2026-10-15</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="O4" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">미확인</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="P4" s="2">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="Q4" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">미확인</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="R4" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">미확인</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="5" spans="1:18" ht="48" customHeight="1">
       <x:c r="A5" s="2" t="s">
         <x:v>109</x:v>
       </x:c>
@@ -7846,6 +8040,46 @@
       </x:c>
       <x:c r="H5" s="3" t="s">
         <x:v>263</x:v>
+      </x:c>
+      <x:c r="I5" s="2">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="J5" s="2">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="K5" s="2">
+        <x:f>I5*J5</x:f>
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="L5" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">우선</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="M5" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">T12 #52014 마커와 첨부, 로컬 사본이 남음. 영향 3은 삭제 요청 정보의 잔존.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="N5" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">2026-10-15</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="O5" s="2">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="P5" s="2">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="Q5" s="2">
+        <x:f>O5*P5</x:f>
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="R5" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">우선</x:t>
+        </x:is>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
docs: add retention fields to the processing sheet
</commit_message>
<xml_diff>
--- a/reports/JY-Audit-Workbook.xlsx
+++ b/reports/JY-Audit-Workbook.xlsx
@@ -138,7 +138,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<x:sst xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="859" uniqueCount="601">
+<x:sst xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="888" uniqueCount="630">
   <x:si>
     <x:t>F-01~F-03 화면·JSON SHA256 수집. users-diff.json은 S05 active True→False만. 명부 이메일 .example.test. 토큰 미저장.</x:t>
   </x:si>
@@ -1954,6 +1954,93 @@
   </x:si>
   <x:si>
     <x:t>종료 계정 비활성+새 로그인 차단</x:t>
+  </x:si>
+  <x:si>
+    <x:t>종료조건</x:t>
+  </x:si>
+  <x:si>
+    <x:t>보존사유</x:t>
+  </x:si>
+  <x:si>
+    <x:t>기산점</x:t>
+  </x:si>
+  <x:si>
+    <x:t>필요기간/판단상태</x:t>
+  </x:si>
+  <x:si>
+    <x:t>파기방법·책임</x:t>
+  </x:si>
+  <x:si>
+    <x:t>예외</x:t>
+  </x:si>
+  <x:si>
+    <x:t>답변 후 추가 문의가 없는 상태. 운영 확인은 하지 않음</x:t>
+  </x:si>
+  <x:si>
+    <x:t>상담 목적. 법령 보관 의무는 원문 확인 전</x:t>
+  </x:si>
+  <x:si>
+    <x:t>상담 종료일. 기산일은 공란</x:t>
+  </x:si>
+  <x:si>
+    <x:t>기간 숫자 없음. 확인 필요</x:t>
+  </x:si>
+  <x:si>
+    <x:t>삭제 버튼만으로 끝나지 않음. 참조, 첨부, 사본, 백업은 따로. 실행 S01, 확인 S02</x:t>
+  </x:si>
+  <x:si>
+    <x:t>P-01과 같음</x:t>
+  </x:si>
+  <x:si>
+    <x:t>유지보수 작업이 끝난 때. 한시 권한은 실행하지 않음</x:t>
+  </x:si>
+  <x:si>
+    <x:t>작업에 필요한 동안. 상담 보유 사유가 아님</x:t>
+  </x:si>
+  <x:si>
+    <x:t>작업 종료. 이번 부여 행은 없음</x:t>
+  </x:si>
+  <x:si>
+    <x:t>계정 비활성과 그룹 회수. PC 사본은 삭제 버튼으로 지워지지 않음. 절차 미완료</x:t>
+  </x:si>
+  <x:si>
+    <x:t>P-04</x:t>
+  </x:si>
+  <x:si>
+    <x:t>실습 증적 보존</x:t>
+  </x:si>
+  <x:si>
+    <x:t>T12 마커와 첨부. 로컬 사본</x:t>
+  </x:si>
+  <x:si>
+    <x:t>고객 보유가 아님</x:t>
+  </x:si>
+  <x:si>
+    <x:t>수행자 로컬</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Zammad의 T12. Git 밖 사본</x:t>
+  </x:si>
+  <x:si>
+    <x:t>증적 고정 후 별도 결정</x:t>
+  </x:si>
+  <x:si>
+    <x:t>시험 증적. 고객 보유 기간과 별도</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2026-10-06 잔존 확인</x:t>
+  </x:si>
+  <x:si>
+    <x:t>기간 숫자 없음. 새 목표일 미정</x:t>
+  </x:si>
+  <x:si>
+    <x:t>미실시. 기한 2026-10-06 경과, 미완료. 승인 S02, 실행 S01</x:t>
+  </x:si>
+  <x:si>
+    <x:t>EX-03. T15는 EX-04이며 파기 대상 아님</x:t>
+  </x:si>
+  <x:si>
+    <x:t>가상 사업에서는 답변 후 추가 문의가 없으면 목적이 끝난 것으로 둔다. 법령 보관 기간 숫자는 확인 필요라 비워 둔다. E01은 미흡이다.</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -2699,17 +2786,21 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="ProcessingTable" displayName="ProcessingTable" ref="A1:H4" totalsRowBorderDxfId="5">
-  <x:autoFilter ref="A1:H4"/>
-  <x:tableColumns count="8">
+<x:table xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="ProcessingTable" displayName="ProcessingTable" ref="A1:L5" totalsRowBorderDxfId="5">
+  <x:autoFilter ref="A1:L5"/>
+  <x:tableColumns count="12">
     <x:tableColumn id="1" name="업무ID" dataDxfId="9"/>
     <x:tableColumn id="2" name="목적" dataDxfId="9"/>
     <x:tableColumn id="3" name="항목" dataDxfId="9"/>
     <x:tableColumn id="4" name="근거" dataDxfId="9"/>
     <x:tableColumn id="5" name="수탁자" dataDxfId="9"/>
     <x:tableColumn id="6" name="저장위치" dataDxfId="9"/>
-    <x:tableColumn id="7" name="보유기준" dataDxfId="9"/>
-    <x:tableColumn id="8" name="파기방법" dataDxfId="9"/>
+    <x:tableColumn id="7" name="종료조건" dataDxfId="9"/>
+    <x:tableColumn id="8" name="보존사유" dataDxfId="9"/>
+    <x:tableColumn id="9" name="기산점" dataDxfId="9"/>
+    <x:tableColumn id="10" name="필요기간/판단상태" dataDxfId="9"/>
+    <x:tableColumn id="11" name="파기방법·책임" dataDxfId="9"/>
+    <x:tableColumn id="12" name="예외" dataDxfId="9"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
@@ -6185,18 +6276,18 @@
     <x:tabColor rgb="ff1e3a5f"/>
     <x:pageSetUpPr autoPageBreaks="1" fitToPage="1"/>
   </x:sheetPr>
-  <x:dimension ref="A1:H4"/>
+  <x:dimension ref="A1:L7"/>
   <x:sheetFormatPr defaultColWidth="8.796875" defaultRowHeight="16.39999999999999857891"/>
   <x:cols>
     <x:col min="1" max="2" width="10" customWidth="1"/>
-    <x:col min="3" max="3" width="15" customWidth="1"/>
+    <x:col min="3" max="3" width="24" customWidth="1"/>
     <x:col min="4" max="4" width="12" customWidth="1"/>
-    <x:col min="5" max="5" width="17" customWidth="1"/>
-    <x:col min="6" max="7" width="16" customWidth="1"/>
-    <x:col min="8" max="8" width="14" customWidth="1"/>
+    <x:col min="5" max="5" width="22" customWidth="1"/>
+    <x:col min="6" max="6" width="24" customWidth="1"/>
+    <x:col min="7" max="12" width="32" customWidth="1"/>
   </x:cols>
   <x:sheetData>
-    <x:row r="1" spans="1:8" ht="28" customHeight="1">
+    <x:row r="1" spans="1:12" ht="28" customHeight="1">
       <x:c r="A1" s="1" t="s">
         <x:v>114</x:v>
       </x:c>
@@ -6216,13 +6307,25 @@
         <x:v>385</x:v>
       </x:c>
       <x:c r="G1" s="1" t="s">
-        <x:v>318</x:v>
+        <x:v>601</x:v>
       </x:c>
       <x:c r="H1" s="1" t="s">
-        <x:v>278</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="2" spans="1:8" ht="36" customHeight="1">
+        <x:v>602</x:v>
+      </x:c>
+      <x:c r="I1" s="1" t="s">
+        <x:v>603</x:v>
+      </x:c>
+      <x:c r="J1" s="1" t="s">
+        <x:v>604</x:v>
+      </x:c>
+      <x:c r="K1" s="1" t="s">
+        <x:v>605</x:v>
+      </x:c>
+      <x:c r="L1" s="1" t="s">
+        <x:v>606</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" spans="1:12" ht="56" customHeight="1">
       <x:c r="A2" s="2" t="s">
         <x:v>362</x:v>
       </x:c>
@@ -6242,13 +6345,25 @@
         <x:v>100</x:v>
       </x:c>
       <x:c r="G2" s="3" t="s">
-        <x:v>143</x:v>
+        <x:v>607</x:v>
       </x:c>
       <x:c r="H2" s="3" t="s">
-        <x:v>36</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="3" spans="1:8" ht="36" customHeight="1">
+        <x:v>608</x:v>
+      </x:c>
+      <x:c r="I2" s="3" t="s">
+        <x:v>609</x:v>
+      </x:c>
+      <x:c r="J2" s="3" t="s">
+        <x:v>610</x:v>
+      </x:c>
+      <x:c r="K2" s="3" t="s">
+        <x:v>611</x:v>
+      </x:c>
+      <x:c r="L2" s="3" t="s">
+        <x:v>421</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" spans="1:12" ht="56" customHeight="1">
       <x:c r="A3" s="2" t="s">
         <x:v>355</x:v>
       </x:c>
@@ -6268,13 +6383,25 @@
         <x:v>137</x:v>
       </x:c>
       <x:c r="G3" s="3" t="s">
-        <x:v>430</x:v>
+        <x:v>612</x:v>
       </x:c>
       <x:c r="H3" s="3" t="s">
-        <x:v>430</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="4" spans="1:8" ht="36" customHeight="1">
+        <x:v>612</x:v>
+      </x:c>
+      <x:c r="I3" s="3" t="s">
+        <x:v>612</x:v>
+      </x:c>
+      <x:c r="J3" s="3" t="s">
+        <x:v>612</x:v>
+      </x:c>
+      <x:c r="K3" s="3" t="s">
+        <x:v>612</x:v>
+      </x:c>
+      <x:c r="L3" s="3" t="s">
+        <x:v>421</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" spans="1:12" ht="56" customHeight="1">
       <x:c r="A4" s="2" t="s">
         <x:v>378</x:v>
       </x:c>
@@ -6294,13 +6421,71 @@
         <x:v>375</x:v>
       </x:c>
       <x:c r="G4" s="3" t="s">
-        <x:v>376</x:v>
+        <x:v>613</x:v>
       </x:c>
       <x:c r="H4" s="3" t="s">
-        <x:v>34</x:v>
+        <x:v>614</x:v>
+      </x:c>
+      <x:c r="I4" s="3" t="s">
+        <x:v>615</x:v>
+      </x:c>
+      <x:c r="J4" s="3" t="s">
+        <x:v>610</x:v>
+      </x:c>
+      <x:c r="K4" s="3" t="s">
+        <x:v>616</x:v>
+      </x:c>
+      <x:c r="L4" s="3" t="s">
+        <x:v>421</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" spans="1:12" ht="56" customHeight="1">
+      <x:c r="A5" s="2" t="s">
+        <x:v>617</x:v>
+      </x:c>
+      <x:c r="B5" s="3" t="s">
+        <x:v>618</x:v>
+      </x:c>
+      <x:c r="C5" s="3" t="s">
+        <x:v>619</x:v>
+      </x:c>
+      <x:c r="D5" s="3" t="s">
+        <x:v>620</x:v>
+      </x:c>
+      <x:c r="E5" s="3" t="s">
+        <x:v>621</x:v>
+      </x:c>
+      <x:c r="F5" s="3" t="s">
+        <x:v>622</x:v>
+      </x:c>
+      <x:c r="G5" s="3" t="s">
+        <x:v>623</x:v>
+      </x:c>
+      <x:c r="H5" s="3" t="s">
+        <x:v>624</x:v>
+      </x:c>
+      <x:c r="I5" s="3" t="s">
+        <x:v>625</x:v>
+      </x:c>
+      <x:c r="J5" s="3" t="s">
+        <x:v>626</x:v>
+      </x:c>
+      <x:c r="K5" s="3" t="s">
+        <x:v>627</x:v>
+      </x:c>
+      <x:c r="L5" s="3" t="s">
+        <x:v>628</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" spans="1:12" ht="56" customHeight="1">
+      <x:c r="A7" s="3" t="s">
+        <x:v>629</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
+  <x:mergeCells count="1">
+    <x:mergeCell ref="A7:L7"/>
+  </x:mergeCells>
   <x:pageMargins left="0.40000000596046447754" right="0.40000000596046447754" top="0.5" bottom="0.5" header="0.5" footer="0.5"/>
   <x:pageSetup paperSize="9" scale="100" firstPageNumber="1" fitToWidth="1" fitToHeight="0" orientation="landscape" usePrinterDefaults="1" blackAndWhite="0" draft="0" useFirstPageNumber="0" horizontalDpi="600" verticalDpi="600" copies="1"/>
   <x:headerFooter differentOddEven="0" differentFirst="0" scaleWithDoc="1" alignWithMargins="1"/>

</xml_diff>